<commit_message>
Add transportation geography analysis, rebuild report and model
New Transport_Geo tab (model now 13 tabs, 166 formulas) and a new
Section 9 subsection (report now 26 pages) estimating student density
by zone from public geography: about 1.4 elementary students per
square mile in the eastern county against 4.6 in the Paris-area zones,
the exact variable KRS 157.370 funds transportation on. Bottom-up
route-mile arithmetic prices closure busing at 51,000 to 147,000
dollars a year, validating the 75,000 to 200,000 planning range and
its 137,500 midpoint, and shows the rebalancing scenario is
transport-neutral to modestly positive. All inputs are labeled
estimates the district's T-1 report and zone map should replace.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -13,12 +13,13 @@
     <sheet name="Closure_Model" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Growth_Model" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Redistricting" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Alternatives" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Debt_Service" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Runway" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Tax_History" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Demographics" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="School_Data" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Transport_Geo" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Alternatives" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Debt_Service" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Runway" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Tax_History" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Demographics" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="School_Data" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -120,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,6 +150,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -516,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -672,24 +675,31 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Student density, route-mile arithmetic, and busing cost scenarios: Transport_Geo tab (backs Section 9).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>CAVEAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Prepared by a former NMES King working alongside Fable 5, an AI research assistant from Anthropic. Estimates are labeled; every figure</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Prepared by a former NMES King working alongside Fable 5, an AI research assistant from Anthropic. Estimates are labeled; every figure</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>should be re-verified against the cited primary sources before formal use. Nothing here alleges misconduct by any official.</t>
         </is>
@@ -701,6 +711,167 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Reserve Runway: Where the Fund Balance Goes Under Each Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Simplified straight-line projection from the FY2025 ending balance; excludes raises, inflation, and one-time items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Projected ending General Fund balance</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>FY2028</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>FY2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Status quo (current drawdown continues)</t>
+        </is>
+      </c>
+      <c r="B5" s="9">
+        <f>GF_Summary!D9-GF_Summary!$D$16</f>
+        <v/>
+      </c>
+      <c r="C5" s="9">
+        <f>B5-GF_Summary!$D$16</f>
+        <v/>
+      </c>
+      <c r="D5" s="9">
+        <f>C5-GF_Summary!$D$16</f>
+        <v/>
+      </c>
+      <c r="E5" s="9">
+        <f>D5-GF_Summary!$D$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>With alternatives package (conservative midpoint; half effect FY2027, full after)</t>
+        </is>
+      </c>
+      <c r="B6" s="9">
+        <f>GF_Summary!D9-GF_Summary!$D$16</f>
+        <v/>
+      </c>
+      <c r="C6" s="9">
+        <f>B6-GF_Summary!$D$16+0.5*Alternatives!$B$21</f>
+        <v/>
+      </c>
+      <c r="D6" s="9">
+        <f>C6-GF_Summary!$D$16+Alternatives!$B$21</f>
+        <v/>
+      </c>
+      <c r="E6" s="9">
+        <f>D6-GF_Summary!$D$16+Alternatives!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Closure only (base-case net saving from FY2027)</t>
+        </is>
+      </c>
+      <c r="B7" s="9">
+        <f>GF_Summary!D9-GF_Summary!$D$16</f>
+        <v/>
+      </c>
+      <c r="C7" s="9">
+        <f>B7-GF_Summary!$D$16+Closure_Model!$B$20</f>
+        <v/>
+      </c>
+      <c r="D7" s="9">
+        <f>C7-GF_Summary!$D$16+Closure_Model!$B$20</f>
+        <v/>
+      </c>
+      <c r="E7" s="9">
+        <f>D7-GF_Summary!$D$16+Closure_Model!$B$20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2% contingency floor (approx., FY2025 basis)</t>
+        </is>
+      </c>
+      <c r="B8" s="18">
+        <f>GF_Summary!$D$14</f>
+        <v/>
+      </c>
+      <c r="C8" s="18">
+        <f>GF_Summary!$D$14</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>GF_Summary!$D$14</f>
+        <v/>
+      </c>
+      <c r="E8" s="18">
+        <f>GF_Summary!$D$14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Reading: the alternatives package restores balance faster than closure, keeps every school open, and adds enrollment revenue rather than risking it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -745,7 +916,7 @@
           <t>2018</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="28" t="n">
         <v>61.3</v>
       </c>
       <c r="G5" s="25" t="inlineStr">
@@ -760,7 +931,7 @@
           <t>2019</t>
         </is>
       </c>
-      <c r="B6" s="26" t="n">
+      <c r="B6" s="28" t="n">
         <v>60.6</v>
       </c>
     </row>
@@ -770,7 +941,7 @@
           <t>2020</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="28" t="n">
         <v>55.9</v>
       </c>
     </row>
@@ -780,7 +951,7 @@
           <t>2021</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="28" t="n">
         <v>54.2</v>
       </c>
     </row>
@@ -790,7 +961,7 @@
           <t>2022</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="28" t="n">
         <v>49.2</v>
       </c>
     </row>
@@ -800,7 +971,7 @@
           <t>2023</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="28" t="n">
         <v>52.4</v>
       </c>
     </row>
@@ -810,7 +981,7 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="28" t="n">
         <v>52.4</v>
       </c>
     </row>
@@ -820,7 +991,7 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="28" t="n">
         <v>52.4</v>
       </c>
     </row>
@@ -830,7 +1001,7 @@
           <t>Tangible/personal rate (recent)</t>
         </is>
       </c>
-      <c r="B14" s="26" t="n">
+      <c r="B14" s="28" t="n">
         <v>64.5</v>
       </c>
     </row>
@@ -840,7 +1011,7 @@
           <t>Motor vehicle rate</t>
         </is>
       </c>
-      <c r="B15" s="26" t="n">
+      <c r="B15" s="28" t="n">
         <v>54.7</v>
       </c>
     </row>
@@ -867,7 +1038,7 @@
           <t>Fayette County</t>
         </is>
       </c>
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="28" t="n">
         <v>80.90000000000001</v>
       </c>
       <c r="G19" s="25" t="inlineStr">
@@ -882,7 +1053,7 @@
           <t>Paris Independent</t>
         </is>
       </c>
-      <c r="B20" s="26" t="n">
+      <c r="B20" s="28" t="n">
         <v>71.5</v>
       </c>
     </row>
@@ -892,7 +1063,7 @@
           <t>Clark County</t>
         </is>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="28" t="n">
         <v>66.8</v>
       </c>
     </row>
@@ -902,7 +1073,7 @@
           <t>Bath County</t>
         </is>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="28" t="n">
         <v>63.4</v>
       </c>
     </row>
@@ -912,7 +1083,7 @@
           <t>Scott County</t>
         </is>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="28" t="n">
         <v>62.9</v>
       </c>
     </row>
@@ -922,7 +1093,7 @@
           <t>Harrison County</t>
         </is>
       </c>
-      <c r="B24" s="26" t="n">
+      <c r="B24" s="28" t="n">
         <v>57.7</v>
       </c>
     </row>
@@ -932,7 +1103,7 @@
           <t>Montgomery County</t>
         </is>
       </c>
-      <c r="B25" s="26" t="n">
+      <c r="B25" s="28" t="n">
         <v>52.5</v>
       </c>
     </row>
@@ -942,7 +1113,7 @@
           <t>Bourbon County</t>
         </is>
       </c>
-      <c r="B26" s="26" t="n">
+      <c r="B26" s="28" t="n">
         <v>52.4</v>
       </c>
     </row>
@@ -952,7 +1123,7 @@
           <t>Nicholas County</t>
         </is>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="28" t="n">
         <v>43.1</v>
       </c>
     </row>
@@ -962,7 +1133,7 @@
           <t>Statewide school average (DOR Table II, 2025)</t>
         </is>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="28" t="n">
         <v>65.13</v>
       </c>
     </row>
@@ -1227,7 +1398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1960,7 +2131,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2254,55 +2425,55 @@
           <t>North Middletown (Bourbon Co.)</t>
         </is>
       </c>
-      <c r="B15" s="26" t="n">
+      <c r="B15" s="28" t="n">
         <v>56.5</v>
       </c>
-      <c r="C15" s="26" t="n">
+      <c r="C15" s="28" t="n">
         <v>63.9</v>
       </c>
-      <c r="D15" s="26" t="n">
+      <c r="D15" s="28" t="n">
         <v>68.59999999999999</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="28" t="n">
         <v>87.90000000000001</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="28" t="n">
         <v>85.8</v>
       </c>
-      <c r="G15" s="26" t="n">
+      <c r="G15" s="28" t="n">
         <v>72.5</v>
       </c>
-      <c r="H15" s="26" t="n">
+      <c r="H15" s="28" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="I15" s="26" t="n">
+      <c r="I15" s="28" t="n">
         <v>56.6</v>
       </c>
-      <c r="J15" s="26" t="n">
+      <c r="J15" s="28" t="n">
         <v>56.9</v>
       </c>
-      <c r="K15" s="26" t="n">
+      <c r="K15" s="28" t="n">
         <v>48.7</v>
       </c>
-      <c r="L15" s="26" t="n">
+      <c r="L15" s="28" t="n">
         <v>49.3</v>
       </c>
-      <c r="M15" s="26" t="n">
+      <c r="M15" s="28" t="n">
         <v>40</v>
       </c>
-      <c r="N15" s="26" t="n">
+      <c r="N15" s="28" t="n">
         <v>50.4</v>
       </c>
-      <c r="P15" s="26" t="n">
+      <c r="P15" s="28" t="n">
         <v>47.7</v>
       </c>
-      <c r="Q15" s="26" t="n">
+      <c r="Q15" s="28" t="n">
         <v>32.1</v>
       </c>
-      <c r="R15" s="26" t="n">
+      <c r="R15" s="28" t="n">
         <v>54.1</v>
       </c>
-      <c r="S15" s="26" t="n">
+      <c r="S15" s="28" t="n">
         <v>58.2</v>
       </c>
     </row>
@@ -2312,58 +2483,58 @@
           <t>Bourbon Central (Bourbon Co.)</t>
         </is>
       </c>
-      <c r="B16" s="26" t="n">
+      <c r="B16" s="28" t="n">
         <v>77.5</v>
       </c>
-      <c r="C16" s="26" t="n">
+      <c r="C16" s="28" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="D16" s="26" t="n">
+      <c r="D16" s="28" t="n">
         <v>72.59999999999999</v>
       </c>
-      <c r="E16" s="26" t="n">
+      <c r="E16" s="28" t="n">
         <v>69.59999999999999</v>
       </c>
-      <c r="F16" s="26" t="n">
+      <c r="F16" s="28" t="n">
         <v>63</v>
       </c>
-      <c r="G16" s="26" t="n">
+      <c r="G16" s="28" t="n">
         <v>74.7</v>
       </c>
-      <c r="H16" s="26" t="n">
+      <c r="H16" s="28" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="I16" s="26" t="n">
+      <c r="I16" s="28" t="n">
         <v>51.8</v>
       </c>
-      <c r="J16" s="26" t="n">
+      <c r="J16" s="28" t="n">
         <v>52.1</v>
       </c>
-      <c r="K16" s="26" t="n">
+      <c r="K16" s="28" t="n">
         <v>30</v>
       </c>
-      <c r="L16" s="26" t="n">
+      <c r="L16" s="28" t="n">
         <v>34</v>
       </c>
-      <c r="M16" s="26" t="n">
+      <c r="M16" s="28" t="n">
         <v>32.8</v>
       </c>
-      <c r="N16" s="26" t="n">
+      <c r="N16" s="28" t="n">
         <v>39.9</v>
       </c>
-      <c r="O16" s="26" t="n">
+      <c r="O16" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="P16" s="26" t="n">
+      <c r="P16" s="28" t="n">
         <v>29.9</v>
       </c>
-      <c r="Q16" s="26" t="n">
+      <c r="Q16" s="28" t="n">
         <v>29</v>
       </c>
-      <c r="R16" s="26" t="n">
+      <c r="R16" s="28" t="n">
         <v>23.8</v>
       </c>
-      <c r="S16" s="26" t="n">
+      <c r="S16" s="28" t="n">
         <v>26.5</v>
       </c>
     </row>
@@ -2373,58 +2544,58 @@
           <t>Cane Ridge (Bourbon Co.)</t>
         </is>
       </c>
-      <c r="B17" s="26" t="n">
+      <c r="B17" s="28" t="n">
         <v>35.2</v>
       </c>
-      <c r="C17" s="26" t="n">
+      <c r="C17" s="28" t="n">
         <v>50.9</v>
       </c>
-      <c r="D17" s="26" t="n">
+      <c r="D17" s="28" t="n">
         <v>56.2</v>
       </c>
-      <c r="E17" s="26" t="n">
+      <c r="E17" s="28" t="n">
         <v>65.5</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="28" t="n">
         <v>34.5</v>
       </c>
-      <c r="G17" s="26" t="n">
+      <c r="G17" s="28" t="n">
         <v>34</v>
       </c>
-      <c r="H17" s="26" t="n">
+      <c r="H17" s="28" t="n">
         <v>49.6</v>
       </c>
-      <c r="I17" s="26" t="n">
+      <c r="I17" s="28" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="26" t="n">
+      <c r="J17" s="28" t="n">
         <v>51.1</v>
       </c>
-      <c r="K17" s="26" t="n">
+      <c r="K17" s="28" t="n">
         <v>57.5</v>
       </c>
-      <c r="L17" s="26" t="n">
+      <c r="L17" s="28" t="n">
         <v>50.4</v>
       </c>
-      <c r="M17" s="26" t="n">
+      <c r="M17" s="28" t="n">
         <v>41.4</v>
       </c>
-      <c r="N17" s="26" t="n">
+      <c r="N17" s="28" t="n">
         <v>38.8</v>
       </c>
-      <c r="O17" s="26" t="n">
+      <c r="O17" s="28" t="n">
         <v>23.8</v>
       </c>
-      <c r="P17" s="26" t="n">
+      <c r="P17" s="28" t="n">
         <v>38.7</v>
       </c>
-      <c r="Q17" s="26" t="n">
+      <c r="Q17" s="28" t="n">
         <v>34.6</v>
       </c>
-      <c r="R17" s="26" t="n">
+      <c r="R17" s="28" t="n">
         <v>35.8</v>
       </c>
-      <c r="S17" s="26" t="n">
+      <c r="S17" s="28" t="n">
         <v>19.3</v>
       </c>
     </row>
@@ -2434,10 +2605,10 @@
           <t>Paris Elementary (Paris Indep.)</t>
         </is>
       </c>
-      <c r="R18" s="26" t="n">
+      <c r="R18" s="28" t="n">
         <v>16.8</v>
       </c>
-      <c r="S18" s="26" t="n">
+      <c r="S18" s="28" t="n">
         <v>12.2</v>
       </c>
     </row>
@@ -2447,10 +2618,10 @@
           <t>Shearer (Clark Co.)</t>
         </is>
       </c>
-      <c r="R19" s="26" t="n">
+      <c r="R19" s="28" t="n">
         <v>30.7</v>
       </c>
-      <c r="S19" s="26" t="n">
+      <c r="S19" s="28" t="n">
         <v>42.3</v>
       </c>
     </row>
@@ -2460,10 +2631,10 @@
           <t>Justice (Clark Co.)</t>
         </is>
       </c>
-      <c r="R20" s="26" t="n">
+      <c r="R20" s="28" t="n">
         <v>43.2</v>
       </c>
-      <c r="S20" s="26" t="n">
+      <c r="S20" s="28" t="n">
         <v>39.3</v>
       </c>
     </row>
@@ -2473,10 +2644,10 @@
           <t>Strode Station (Clark Co.)</t>
         </is>
       </c>
-      <c r="R21" s="26" t="n">
+      <c r="R21" s="28" t="n">
         <v>43.2</v>
       </c>
-      <c r="S21" s="26" t="n">
+      <c r="S21" s="28" t="n">
         <v>34.2</v>
       </c>
     </row>
@@ -2486,10 +2657,10 @@
           <t>Conkwright (Clark Co.)</t>
         </is>
       </c>
-      <c r="R22" s="26" t="n">
+      <c r="R22" s="28" t="n">
         <v>15.6</v>
       </c>
-      <c r="S22" s="26" t="n">
+      <c r="S22" s="28" t="n">
         <v>17.5</v>
       </c>
     </row>
@@ -2499,10 +2670,10 @@
           <t>Northview (Montgomery Co.)</t>
         </is>
       </c>
-      <c r="R23" s="26" t="n">
+      <c r="R23" s="28" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="S23" s="26" t="n">
+      <c r="S23" s="28" t="n">
         <v>68.90000000000001</v>
       </c>
     </row>
@@ -2512,10 +2683,10 @@
           <t>Mapleton (Montgomery Co.)</t>
         </is>
       </c>
-      <c r="R24" s="26" t="n">
+      <c r="R24" s="28" t="n">
         <v>65.90000000000001</v>
       </c>
-      <c r="S24" s="26" t="n">
+      <c r="S24" s="28" t="n">
         <v>65.09999999999999</v>
       </c>
     </row>
@@ -2525,7 +2696,7 @@
           <t>Nicholas County Elementary (Nicholas Co.)</t>
         </is>
       </c>
-      <c r="R25" s="26" t="n">
+      <c r="R25" s="28" t="n">
         <v>15.9</v>
       </c>
       <c r="T25" s="2" t="inlineStr">
@@ -2635,7 +2806,7 @@
           <t>Composite: economically disadvantaged students</t>
         </is>
       </c>
-      <c r="B34" s="26" t="n">
+      <c r="B34" s="28" t="n">
         <v>57.1</v>
       </c>
     </row>
@@ -2645,7 +2816,7 @@
           <t>Composite: female students</t>
         </is>
       </c>
-      <c r="B35" s="26" t="n">
+      <c r="B35" s="28" t="n">
         <v>85.7</v>
       </c>
     </row>
@@ -2655,7 +2826,7 @@
           <t>Composite: male students</t>
         </is>
       </c>
-      <c r="B36" s="26" t="n">
+      <c r="B36" s="28" t="n">
         <v>28.8</v>
       </c>
     </row>
@@ -4626,6 +4797,544 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Transportation and Geography: Density, Route Miles, and What Closure Adds</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Estimates built from public geography (census counts, county land area, highway distances). The district's annual T-1 transportation report, zone map, and geocoded counts are the authoritative dataset; releasing them is a records ask.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>GEOGRAPHY AND STUDENT DENSITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Bourbon County land area (square miles)</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>290</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>U.S. Census: 289.7 land square miles</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Paris city population, 2020</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>10171</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2020 Census</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Millersburg population, 2020</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>747</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>2020 Census</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>North Middletown population, 2020</t>
+        </is>
+      </c>
+      <c r="B8" s="24">
+        <f>Demographics!B29</f>
+        <v/>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Demographics tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>NMES zone share of county area</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Eastern portion of the county; replace with the district's actual zone map</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>NMES zone area (sq mi)</t>
+        </is>
+      </c>
+      <c r="B10" s="26">
+        <f>B5*B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Paris-area zones (sq mi)</t>
+        </is>
+      </c>
+      <c r="B11" s="26">
+        <f>B5-B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>NMES elementary students</t>
+        </is>
+      </c>
+      <c r="B12" s="24">
+        <f>Assumptions!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Paris-area elementary students</t>
+        </is>
+      </c>
+      <c r="B13" s="24">
+        <f>Redistricting!B8+Redistricting!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Students per square mile, NMES zone</t>
+        </is>
+      </c>
+      <c r="B14" s="20">
+        <f>B12/B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Students per square mile, Paris-area zones</t>
+        </is>
+      </c>
+      <c r="B15" s="20">
+        <f>B13/B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Students per square mile, district elementary overall</t>
+        </is>
+      </c>
+      <c r="B16" s="20">
+        <f>(B12+B13)/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>State law (KRS 157.370) funds transportation on transported pupils per square mile: low density earns a higher per-pupil allotment because it costs more to serve. The statutory calculation has been funded below its own formula in every budget since 2005.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>WHAT CLOSURE ADDS: ROUTE-MILE ARITHMETIC (yellow = replace with district T-1 data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Share of NMES students riding the bus</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Riders</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>ROUND(B20*B12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Rural routes serving NMES today</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Added distance to the Paris schools, one way (miles)</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>US 460, North Middletown to Paris</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Added bus-miles per route per day (out and back, AM and PM)</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>B23*4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>School days per year</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Added bus-miles per year</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>B22*B24*B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Marginal cost per bus-mile, low</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Fuel, maintenance, driver time; replace with district cost data</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Marginal cost per bus-mile, high</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Added cost, mileage basis, low</t>
+        </is>
+      </c>
+      <c r="B29" s="9">
+        <f>B26*B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Added cost, mileage basis, high</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>B26*B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Additional buses if route tiers break (high case)</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>All-in cost per additional bus-year</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Bottom-up added busing cost, low</t>
+        </is>
+      </c>
+      <c r="B33" s="23">
+        <f>B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Bottom-up added busing cost, high</t>
+        </is>
+      </c>
+      <c r="B34" s="22">
+        <f>B30+B31*B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Report's planning range (Closure_Model offset basis)</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Between $75,000 and $200,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
+        <is>
+          <t>The bottom-up estimate lands inside the planning range; the $137,500 midpoint used in the Closure_Model stands. Note what closure does not remove: every square mile of the eastern county stays in the coverage area, with longer rides on it, roughly 15 to 20 added minutes each way on US 460.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>WHAT REBALANCING CHANGES (Redistricting tab scenario)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Students rezoned to NMES</t>
+        </is>
+      </c>
+      <c r="B39" s="24">
+        <f>Redistricting!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Stem miles saved per affected route, one way</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Rezoned families live closer to NMES than to their assigned school</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Affected routes</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Bus-miles saved per year</t>
+        </is>
+      </c>
+      <c r="B42" s="11">
+        <f>B41*B40*4*B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Transport saving, low</t>
+        </is>
+      </c>
+      <c r="B43" s="9">
+        <f>B42*B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Transport saving, high</t>
+        </is>
+      </c>
+      <c r="B44" s="9">
+        <f>B42*B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Rebalancing is transport-neutral to modestly positive, the opposite sign of closure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>DISTRICT-WIDE CONTEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Transportation expense, FY2025</t>
+        </is>
+      </c>
+      <c r="B48" s="18">
+        <f>Assumptions!B42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Average Daily Attendance, FY2025</t>
+        </is>
+      </c>
+      <c r="B49" s="28" t="n">
+        <v>2242.5</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Transportation cost per student in attendance</t>
+        </is>
+      </c>
+      <c r="B50" s="9">
+        <f>B48/B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Optimization potential at 5 to 10 percent (Alternatives menu)</t>
+        </is>
+      </c>
+      <c r="B51" s="18">
+        <f>Assumptions!B42*Assumptions!B43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr"/>
+      <c r="B52" s="18">
+        <f>Assumptions!B42*Assumptions!B44</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4960,7 +5669,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5297,7 +6006,7 @@
           <t>Average Daily Attendance, FY2025 (SEEK basis)</t>
         </is>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="28" t="n">
         <v>2242.5</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -5354,7 +6063,7 @@
           <t>Annual restricted margin available for new debt (illustrative)</t>
         </is>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="29">
         <f>B23*B24+B25-B26</f>
         <v/>
       </c>
@@ -5418,167 +6127,6 @@
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>the official statement, and the bonding potential statement all public.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Reserve Runway: Where the Fund Balance Goes Under Each Path</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Simplified straight-line projection from the FY2025 ending balance; excludes raises, inflation, and one-time items.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="17" t="inlineStr">
-        <is>
-          <t>Projected ending General Fund balance</t>
-        </is>
-      </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>FY2026</t>
-        </is>
-      </c>
-      <c r="C4" s="17" t="inlineStr">
-        <is>
-          <t>FY2027</t>
-        </is>
-      </c>
-      <c r="D4" s="17" t="inlineStr">
-        <is>
-          <t>FY2028</t>
-        </is>
-      </c>
-      <c r="E4" s="17" t="inlineStr">
-        <is>
-          <t>FY2029</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Status quo (current drawdown continues)</t>
-        </is>
-      </c>
-      <c r="B5" s="9">
-        <f>GF_Summary!D9-GF_Summary!$D$16</f>
-        <v/>
-      </c>
-      <c r="C5" s="9">
-        <f>B5-GF_Summary!$D$16</f>
-        <v/>
-      </c>
-      <c r="D5" s="9">
-        <f>C5-GF_Summary!$D$16</f>
-        <v/>
-      </c>
-      <c r="E5" s="9">
-        <f>D5-GF_Summary!$D$16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>With alternatives package (conservative midpoint; half effect FY2027, full after)</t>
-        </is>
-      </c>
-      <c r="B6" s="9">
-        <f>GF_Summary!D9-GF_Summary!$D$16</f>
-        <v/>
-      </c>
-      <c r="C6" s="9">
-        <f>B6-GF_Summary!$D$16+0.5*Alternatives!$B$21</f>
-        <v/>
-      </c>
-      <c r="D6" s="9">
-        <f>C6-GF_Summary!$D$16+Alternatives!$B$21</f>
-        <v/>
-      </c>
-      <c r="E6" s="9">
-        <f>D6-GF_Summary!$D$16+Alternatives!$B$21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Closure only (base-case net saving from FY2027)</t>
-        </is>
-      </c>
-      <c r="B7" s="9">
-        <f>GF_Summary!D9-GF_Summary!$D$16</f>
-        <v/>
-      </c>
-      <c r="C7" s="9">
-        <f>B7-GF_Summary!$D$16+Closure_Model!$B$20</f>
-        <v/>
-      </c>
-      <c r="D7" s="9">
-        <f>C7-GF_Summary!$D$16+Closure_Model!$B$20</f>
-        <v/>
-      </c>
-      <c r="E7" s="9">
-        <f>D7-GF_Summary!$D$16+Closure_Model!$B$20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>2% contingency floor (approx., FY2025 basis)</t>
-        </is>
-      </c>
-      <c r="B8" s="18">
-        <f>GF_Summary!$D$14</f>
-        <v/>
-      </c>
-      <c r="C8" s="18">
-        <f>GF_Summary!$D$14</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>GF_Summary!$D$14</f>
-        <v/>
-      </c>
-      <c r="E8" s="18">
-        <f>GF_Summary!$D$14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>Reading: the alternatives package restores balance faster than closure, keeps every school open, and adds enrollment revenue rather than risking it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reframe scenario 1 as the districtwide status quo
Plan 1 is now labeled the districtwide status quo across the report,
site, and model Scenarios tab, with text making explicit that the
deficit is a districtwide problem NMES did not cause and that the
reserve drawdown happens with or without the school.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -933,7 +933,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>1. Keep NMES open, current trajectory</t>
+          <t>1. Districtwide status quo (change nothing anywhere)</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
@@ -950,7 +950,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>No decisions; reserves cross below zero on the straight line and the gap remains unaddressed</t>
+          <t>No decisions; the districtwide gap, which NMES did not cause, drains reserves below zero with or without the school</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consolidate rebalance-and-grow into the districtwide recovery plan
The scenarios comparison now shows three complete plans; rebalancing
and growing NMES ($140,000 to $225,000 a year) is named as one line
inside the recovery plan's menu across the report, site, and model.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -879,7 +879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -982,57 +982,32 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>3. Keep NMES open, rebalance and grow</t>
+          <t>3. Districtwide recovery plan (menu plus levy; includes rebalancing and growing NMES)</t>
         </is>
       </c>
       <c r="B7" s="18">
-        <f>Redistricting!B30</f>
+        <f>Alternatives!B21</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>GF_Summary!D9-4*GF_Summary!D16+3*Redistricting!B30</f>
+        <f>Runway!E6</f>
         <v/>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Minimal (boundary process)</t>
+          <t>Varies by measure</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Board boundary action and HB 563 recruitment; academic upside; does not close the gap alone</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>4. Districtwide recovery plan (menu plus levy)</t>
-        </is>
-      </c>
-      <c r="B8" s="18">
-        <f>Alternatives!B21</f>
-        <v/>
-      </c>
-      <c r="C8" s="9">
-        <f>Runway!E6</f>
-        <v/>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Varies by measure</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Revenue votes, administrative rollback, and implementation discipline; keeps every school open</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>Reading: the question before the board is not closure versus no closure. It is which complete plan produces the best verified five-year result. Plan 2 buys roughly one extra year of runway; Plan 4 restores balance. Plans 3 and 4 combine.</t>
+          <t>Revenue votes, administrative rollback, boundary action and HB 563 recruitment, implementation discipline; every school stays open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Reading: the question before the board is not closure versus no closure. It is which complete plan produces the best verified five-year result. Plan 2 buys roughly one extra year of runway; Plan 3 restores balance while keeping every school open. The rebalance-and-grow scenario (Redistricting tab) is one line inside Plan 3's menu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
State current receiving capacities as 549 and 422
Bourbon Central's rating today is 549, the to-become capacity its
2021 plan listed with its addition; Cane Ridge remains 422. The
squeeze math now leads with those ratings everywhere: 90 open at
Bourbon Central, 31 over at Cane Ridge, net 59 uncommitted seats for
128 children, with the 2021 plan's as-printed 521 kept as a
sensitivity (net 31). Figure 12's capacity lines, the site card and
banner, Question 3, the exec summary, and the model's Facility_Plans
tab all updated; validation checks pin the new figures.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -3109,7 +3109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Plan lists a to-become capacity of 549 after an addition not yet built</t>
+          <t>Rating today is 549, the plan's to-become capacity with its addition</t>
         </is>
       </c>
     </row>
@@ -3188,18 +3188,18 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>RECEIVING CAPACITY TODAY (2021 plan capacities vs 2024-25 enrollment)</t>
+          <t>RECEIVING CAPACITY TODAY (current ratings vs 2024-25 enrollment)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Bourbon Central open seats at rated 521</t>
+          <t>Bourbon Central open seats at its current rated 549</t>
         </is>
       </c>
       <c r="B13" s="11">
-        <f>E7-Redistricting!B8</f>
+        <f>549-Redistricting!B8</f>
         <v/>
       </c>
     </row>
@@ -3250,11 +3250,11 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Net seats even after Bourbon Central's planned (unbuilt) expansion to 549</t>
+          <t>Sensitivity: net seats at the 2021 plan's as-printed 521 for Bourbon Central</t>
         </is>
       </c>
       <c r="B18" s="11">
-        <f>549-Redistricting!B8-B14</f>
+        <f>E7-Redistricting!B8-B14</f>
         <v/>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>Reading: the plans rate the receiving schools at 521 and 422 seats. At current enrollment that is 62 open at Bourbon Central and 31 over at Cane Ridge, a net 31 uncommitted seats for 128 children. NMES renovation needs were priced in 2013 and re-priced higher in 2021, each time scheduled behind other work. Its rated capacity fell 198 to 174 between the same two plans while its enrollment fell 169 to 128.</t>
+          <t>Reading: the receiving schools' current ratings are 549 (Bourbon Central) and 422 (Cane Ridge). At current enrollment that is 90 open at Bourbon Central and 31 over at Cane Ridge, a net 59 uncommitted seats for 128 children (net 31 at the 2021 plan's as-printed 521). NMES renovation needs were priced in 2013 and re-priced higher in 2021, each time scheduled behind other work. Its rated capacity fell 198 to 174 between the same two plans while its enrollment fell 169 to 128.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Treat 549 as Bourbon Central's rated capacity throughout
State the receiving capacities plainly as 549 and 422, note simply
that 549 reflects the addition in the 2021 plan, and drop the
as-printed-521 sensitivity framing from the report, site, and model.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -3109,7 +3109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Rating today is 549, the plan's to-become capacity with its addition</t>
+          <t>Rated capacity 549, reflecting the addition in the 2021 plan</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3195,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Bourbon Central open seats at its current rated 549</t>
+          <t>Bourbon Central open seats at rated 549</t>
         </is>
       </c>
       <c r="B13" s="11">
@@ -3247,17 +3247,6 @@
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Sensitivity: net seats at the 2021 plan's as-printed 521 for Bourbon Central</t>
-        </is>
-      </c>
-      <c r="B18" s="11">
-        <f>E7-Redistricting!B8-B14</f>
-        <v/>
-      </c>
-    </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -3339,7 +3328,7 @@
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>Reading: the receiving schools' current ratings are 549 (Bourbon Central) and 422 (Cane Ridge). At current enrollment that is 90 open at Bourbon Central and 31 over at Cane Ridge, a net 59 uncommitted seats for 128 children (net 31 at the 2021 plan's as-printed 521). NMES renovation needs were priced in 2013 and re-priced higher in 2021, each time scheduled behind other work. Its rated capacity fell 198 to 174 between the same two plans while its enrollment fell 169 to 128.</t>
+          <t>Reading: the receiving schools' rated capacities are 549 (Bourbon Central) and 422 (Cane Ridge). At current enrollment that is 90 open at Bourbon Central and 31 over at Cane Ridge, a net 59 uncommitted seats for 128 children. NMES renovation needs were priced in 2013 and re-priced higher in 2021, each time scheduled behind other work. Its rated capacity fell 198 to 174 between the same two plans while its enrollment fell 169 to 128.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct the biennium scheduling claim and adopt tone fixes
- The 2021 plan schedules NMES's life-safety and accessibility work
  ($642,660) within the 2022-24 biennium and only the $3.62M major
  renovation after it; the report, site, and model now say exactly
  that instead of "every dollar after the biennium"
- Fix the stale "Four Complete Plans" title on the model's Scenarios
  tab (three plans)
- Tone: rated capacity is "shaped through room assignments and
  planning submissions" and raised "through the same process";
  "proposed for reclassification" replaces "slated for closure";
  "no public recruitment program has marketed" drops the absolute;
  the high school row states the rating rise, not "expansion built"
- Add the preschool center row (over capacity in both plans) to the
  site's facility-plans table

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -894,7 +894,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Four Complete Plans, Compared (illustrative five-year view)</t>
+          <t>Three Complete Plans, Compared (illustrative five-year view)</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Expansion built; CTC addition was the 2022-24 in-biennium priority</t>
+          <t>Rating rose 637 to 704 between plans; the CTC addition was the 2022-24 in-biennium priority</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>All scheduled after the 2022-24 biennium; the in-biennium priority was the HS Career &amp; Technical Center</t>
+          <t>Life safety and accessibility ($642,660) within the 2022-24 biennium; the $3.62M major renovation after it; the biennium's headline priority was the HS Career &amp; Technical Center</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>Reading: the receiving schools' rated capacities are 549 (Bourbon Central) and 422 (Cane Ridge). At current enrollment that is 90 open at Bourbon Central and 31 over at Cane Ridge, a net 59 uncommitted seats for 128 children. NMES renovation needs were priced in 2013 and re-priced higher in 2021, each time scheduled behind other work. Its rated capacity fell 198 to 174 between the same two plans while its enrollment fell 169 to 128.</t>
+          <t>Reading: the receiving schools' rated capacities are 549 (Bourbon Central) and 422 (Cane Ridge). At current enrollment that is 90 open at Bourbon Central and 31 over at Cane Ridge, a net 59 uncommitted seats for 128 children. NMES's major renovation was priced in 2013 and re-priced higher in 2021, each time scheduled after the then-current biennium. Its rated capacity fell 198 to 174 between the same two plans while its enrollment fell 169 to 128.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the multi-age reorganization lever from the analysis
Drop the NMES multi-age reorganization option everywhere it appeared:
the Alternatives menu line in the model, the Figure 14 table note, the
grow-narrative option list, the sustainability-committee charge, and
the closure staffing-reconciliation sentence (which no longer needs it,
the three-to-five-position range now stands on the receiving-schools
judgment alone). Combining grades would have cut against the school's
small-class strength, so it does not belong in the keep-open case.

The raw alternatives sum falls to about $1.6 to $2.8 million; the
published $1.1 to $2.1 million band and the recovery-plan scenario are
unchanged (the band was already a conservative haircut, now described
as such rather than pinned to a fraction). Model holds at 193 formulas;
suite at 96/35/14; Version 2.6 unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -7141,7 +7141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -7486,123 +7486,95 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>NMES multi-age reorganization</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>170000</v>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>255000</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Six or seven sections instead of nine, via attrition</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Cost reduction</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Medium; needs a staffing and grade-band plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Total identified (ranges overlap; not additive to the penny)</t>
         </is>
       </c>
-      <c r="B15" s="24">
-        <f>SUM(B4:B14)</f>
-        <v/>
-      </c>
-      <c r="C15" s="24">
-        <f>SUM(C4:C14)</f>
-        <v/>
+      <c r="B14" s="24">
+        <f>SUM(B4:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="24">
+        <f>SUM(C4:C13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>COMPARISON</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>COMPARISON</t>
-        </is>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Package midpoint (raw sum of ranges)</t>
+        </is>
+      </c>
+      <c r="B17" s="9">
+        <f>(B14+C14)/2</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Package midpoint (raw sum of ranges)</t>
-        </is>
-      </c>
-      <c r="B18" s="9">
-        <f>(B15+C15)/2</f>
-        <v/>
+          <t>Conservative combined estimate, low (haircut for overlap)</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>1100000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Conservative combined estimate, low (haircut for overlap)</t>
+          <t>Conservative combined estimate, high</t>
         </is>
       </c>
       <c r="B19" s="14" t="n">
-        <v>1100000</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Conservative combined estimate, high</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="n">
-        <v>2100000</v>
+          <t>Conservative midpoint (used in Runway sheet)</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>(B18+B19)/2</f>
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Conservative midpoint (used in Runway sheet)</t>
-        </is>
-      </c>
-      <c r="B21" s="9">
-        <f>(B19+B20)/2</f>
+          <t>Average annual GF drawdown (FY2024-25)</t>
+        </is>
+      </c>
+      <c r="B21" s="18">
+        <f>GF_Summary!D16</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Average annual GF drawdown (FY2024-25)</t>
+          <t>Closure net saving (base case)</t>
         </is>
       </c>
       <c r="B22" s="18">
-        <f>GF_Summary!D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Closure net saving (base case)</t>
-        </is>
-      </c>
-      <c r="B23" s="18">
         <f>Closure_Model!B20</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>Reading: raw row sums run about $1.7M to $3.0M; the published $1.1M to $2.1M band takes roughly two thirds of them as a haircut for overlap and implementation risk. Coverage is reported against both yardsticks: the $2.65M structural gap before transfers and the roughly $1.15M net drawdown after transfers (Closure_Model rows 21 and 35 carry both for closure).</t>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Reading: raw row sums run about $1.6M to $2.8M; the published $1.1M to $2.1M band applies a conservative haircut for overlap and implementation risk. Coverage is reported against both yardsticks: the $2.65M structural gap before transfers and the roughly $1.15M net drawdown after transfers (Closure_Model rows 21 and 35 carry both for closure).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add bonding story: $14M plan analysis, funding levers, unaudited FY2026 close
Site, report (v2.6, 34pp), and model Debt_Service tab gain the $14M
general fund bond analysis, savings-to-bond-capacity scenarios, the
three funding levers, and the FY2026 KDE Budget Monitoring Tool close
(labeled unaudited, with the $1.57M miscellaneous-receipt caveat).
June 2026 financial packet archived. 13 new test checks; suite green.

Staged on branch only; not merged to main pending review.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,6 +157,7 @@
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2955,7 +2956,7 @@
           <t>Subject</t>
         </is>
       </c>
-      <c r="B34" s="31" t="inlineStr">
+      <c r="B34" s="32" t="inlineStr">
         <is>
           <t>NMES</t>
         </is>
@@ -4031,7 +4032,7 @@
           <t>Net uncommitted seats at both receiving schools</t>
         </is>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="33">
         <f>B13-B14</f>
         <v/>
       </c>
@@ -4053,7 +4054,7 @@
           <t>Shortfall if closure proceeds today</t>
         </is>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="33">
         <f>B16-B15</f>
         <v/>
       </c>
@@ -4229,7 +4230,7 @@
           <t>Paper seats added at the receiving schools, with the draft's new-construction sections reading None</t>
         </is>
       </c>
-      <c r="B33" s="32">
+      <c r="B33" s="33">
         <f>D30+D31</f>
         <v/>
       </c>
@@ -4240,7 +4241,7 @@
           <t>NMES fill rate even at the draft's own 154 rating</t>
         </is>
       </c>
-      <c r="B34" s="33">
+      <c r="B34" s="34">
         <f>B32/C32</f>
         <v/>
       </c>
@@ -4465,7 +4466,7 @@
           <t>Net receiving seats at the slides' own capacities (499 and 397)</t>
         </is>
       </c>
-      <c r="B50" s="32">
+      <c r="B50" s="33">
         <f>(499-Redistricting!B8)-(Redistricting!B9-397)</f>
         <v/>
       </c>
@@ -7589,7 +7590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8044,6 +8045,426 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>THE $14 MILLION PLAN (JULY 15, 2026 PLANNING COMMITTEE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Stated plan: free up $800,000 to $1,000,000 a year of operating money to bond $14 million</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Proposed bond amount</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="n">
+        <v>14000000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Assumed interest rate</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Assumed term, years</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Annual debt service on the proposed bond</t>
+        </is>
+      </c>
+      <c r="B42" s="30">
+        <f>B39*B40/(1-(1+B40)^-B41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="21" t="inlineStr">
+        <is>
+          <t>The payment equals the operating money the plan frees up: the school's claimed cost becomes the mortgage</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>WHAT EACH SAVINGS ESTIMATE COULD ACTUALLY BOND</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Bond principal supported = annual savings x present-value annuity factor at the rate and term above</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>District's own KDE-filed excess cost of NMES vs peer elementaries</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n">
+        <v>121220</v>
+      </c>
+      <c r="C46" s="9">
+        <f>B46*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="F46" s="21" t="inlineStr">
+        <is>
+          <t>Matches the closure model's worst case</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Closure model default net saving</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="n">
+        <v>361240</v>
+      </c>
+      <c r="C47" s="9">
+        <f>B47*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="F47" s="21" t="inlineStr">
+        <is>
+          <t>Closure_Model tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Closure model best case</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="n">
+        <v>725000</v>
+      </c>
+      <c r="C48" s="9">
+        <f>B48*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="F48" s="21" t="inlineStr">
+        <is>
+          <t>Closure_Model tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Administration's claim, July 15, 2026</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="n">
+        <v>900000</v>
+      </c>
+      <c r="C49" s="9">
+        <f>B49*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="F49" s="21" t="inlineStr">
+        <is>
+          <t>Unpublished derivation; reconcile with KDE-filed school-level spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Only the administration's own number reaches $14 million. The audited excess cost supports about $1.6 million.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>DISTRICT-PAID DEBT SERVICE SCHEDULE (FY2025 AUDIT, NOTE 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Payments fall as the 2013, 2016, and 2020 series retire; this falling schedule is the room a wrap-around structure fills</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>FY2026</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="n">
+        <v>1578700</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="n">
+        <v>1575060</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>FY2028</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="n">
+        <v>1578719</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>FY2029</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="n">
+        <v>1577258</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>FY2030</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="n">
+        <v>1578340</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>FY2031-35 average</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="n">
+        <v>1321112</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>FY2036-40 average</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="n">
+        <v>398915</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>FY2041-45 average</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="n">
+        <v>260708</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>THE LEVERS THAT DO NOT CLOSE A SCHOOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Remaining restricted capacity (FY2024 audit $23.5M less local share of the 2024 issue, approximate)</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="n">
+        <v>17600000</v>
+      </c>
+      <c r="F64" s="21" t="inlineStr">
+        <is>
+          <t>Exact figure is the fiscal agent's bonding potential statement; demand it</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Certified real and personal property assessment, FY2025</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="n">
+        <v>1843569625</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>Recallable nickel yield per year (5 cents per $100)</t>
+        </is>
+      </c>
+      <c r="B66" s="9">
+        <f>B65*0.0005</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Bonds a nickel supports before state FSPK equalization</t>
+        </is>
+      </c>
+      <c r="B67" s="9">
+        <f>B66*(1-(1+B40)^-B41)/B40</f>
+        <v/>
+      </c>
+      <c r="F67" s="21" t="inlineStr">
+        <is>
+          <t>FSPK equalization adds state dollars on top; KDE's tables set the amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>SFCC offers of assistance, typical cycle</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="n">
+        <v>1750000</v>
+      </c>
+      <c r="F68" s="21" t="inlineStr">
+        <is>
+          <t>State already pays $1,568,809 of current principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>FY2026 YEAR-END, DISTRICT'S OWN KDE BUDGET MONITORING TOOL (UNAUDITED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>June 2026 financial packet, board agenda July 16, 2026; MUNIS run July 15, 2026. Audit will finalize these figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>General Fund revenue, FY2026 actual (excludes carryforward and on-behalf)</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="n">
+        <v>22103877</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>General Fund expenditures, FY2026 actual</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="n">
+        <v>22477866</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Net General Fund change, FY2026 (unaudited)</t>
+        </is>
+      </c>
+      <c r="B74" s="30">
+        <f>B72-B73</f>
+        <v/>
+      </c>
+      <c r="F74" s="21" t="inlineStr">
+        <is>
+          <t>Compare net changes of -$1,065,657 in FY2024 and -$1,225,465 in FY2025 (audited)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Revenues over budget per the monitoring tool</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="n">
+        <v>2225835</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Salaries under budget per the monitoring tool</t>
+        </is>
+      </c>
+      <c r="B76" s="8" t="n">
+        <v>587592</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Salaries below FY2025 actuals</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="n">
+        <v>223974</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Caveat: miscellaneous revenue budgeted at zero, received</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="n">
+        <v>1567829</v>
+      </c>
+      <c r="F78" s="21" t="inlineStr">
+        <is>
+          <t>If one-time, the underlying gap is about $1.9 million; the district should identify this receipt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add balanced-budget bonding capacity scenario
Debt_Service tab: two-case scenario (conservative $1.9M gap vs
unaudited FY2026 $373,989 gap) balancing operations first from
three years of 4 percent levy increments plus $1M recurring cost
reductions, then capitalizing the remainder plus the recallable
nickel. Site and report reference the $30M/$50M range.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -7590,7 +7590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8465,6 +8465,202 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>SCENARIO: BALANCE THE BUDGET AND EXPAND BONDING CAPACITY, NO CLOSURE</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Two cases differ only in the operating gap assumed. Conservative treats the FY2026 $1.57M receipt as one-time;</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>trend uses the unaudited FY2026 net change. Operations are balanced first; only the remainder services debt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="17" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>FY2026 trend</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Operating gap to close first</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="C84" s="8" t="n">
+        <v>373989</v>
+      </c>
+      <c r="F84" s="21" t="inlineStr">
+        <is>
+          <t>Editable. $1.9M = FY2026 result excluding the unidentified receipt; $373,989 = FY2026 unaudited net change</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>New recurring revenue: 4 percent levy taken three years running</t>
+        </is>
+      </c>
+      <c r="B85" s="18">
+        <f>Tax_History!B32*(1.04^3-1)</f>
+        <v/>
+      </c>
+      <c r="C85" s="18">
+        <f>Tax_History!B32*(1.04^3-1)</f>
+        <v/>
+      </c>
+      <c r="F85" s="21" t="inlineStr">
+        <is>
+          <t>Same base and compounding as the levy tab; year 1 is $313,162, year 3 cumulative $977,568</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Recurring cost reductions, not from closing a school</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C86" s="8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F86" s="21" t="inlineStr">
+        <is>
+          <t>Editable. For scale from the FY2025 audit: district administration grew $221K in one year, salaries fell $224K through attrition, spending ran $859K under budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Operating room left for debt service after the budget balances</t>
+        </is>
+      </c>
+      <c r="B87" s="9">
+        <f>MAX(0,B85+B86-B84)</f>
+        <v/>
+      </c>
+      <c r="C87" s="9">
+        <f>MAX(0,C85+C86-C84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>General-fund bond capacity from that room</t>
+        </is>
+      </c>
+      <c r="B88" s="9">
+        <f>B87*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="C88" s="9">
+        <f>C87*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Recallable nickel yield, restricted, before FSPK equalization</t>
+        </is>
+      </c>
+      <c r="B89" s="9">
+        <f>B65*0.0005</f>
+        <v/>
+      </c>
+      <c r="C89" s="9">
+        <f>B65*0.0005</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Bond capacity from the nickel</t>
+        </is>
+      </c>
+      <c r="B90" s="9">
+        <f>B89*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="C90" s="9">
+        <f>C89*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Existing unused restricted capacity, approximate</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="n">
+        <v>17600000</v>
+      </c>
+      <c r="C91" s="8" t="n">
+        <v>17600000</v>
+      </c>
+      <c r="F91" s="21" t="inlineStr">
+        <is>
+          <t>FY2024 audit $23.5M less local share of the 2024 issue; fiscal agent's statement is the authority</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="22" t="inlineStr">
+        <is>
+          <t>Total capacity available without closing a school</t>
+        </is>
+      </c>
+      <c r="B92" s="24">
+        <f>B88+B90+B91</f>
+        <v/>
+      </c>
+      <c r="C92" s="24">
+        <f>C88+C90+C91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Roughly $30.6 million in the conservative case and $50.4 million on the FY2026 trend, with the budget balanced</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>first in both. The administration's plan reaches $32 million at face value and leaves the deficit in place.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Correct nickel analysis: Bourbon already levies a recallable nickel
KDE SEEK District Payment Schedules (FY2026 final, FY2027 forecast)
show a nonzero Recallable Nickel state equalization amount for
district 041, which the schedule pays only on levied nickels. The
site, report, and model previously described the recallable nickel
as an untaken option. Corrected: the nickel is levied and its local
yield already sits inside the building-fund stream; the genuinely
new element is state equalization of $276,246 a year (FY2027
schedule; $55,515 partial FY2026), which is additive to the FY2024
audit's bonding potential. Balanced-budget scenario recomputed:
$22.2M conservative / $42.1M trend (was $30.6M / $50.4M).
Correction noted in the site's own text.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -7590,7 +7590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8331,331 +8331,355 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Recallable nickel yield per year (5 cents per $100)</t>
-        </is>
-      </c>
-      <c r="B66" s="9">
-        <f>B65*0.0005</f>
-        <v/>
+          <t>Recallable nickel status: ALREADY LEVIED, inside the existing rate</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>levied</t>
+        </is>
+      </c>
+      <c r="F66" s="21" t="inlineStr">
+        <is>
+          <t>KDE SEEK District Payment Schedules show a nonzero Recallable Nickel state amount for Bourbon (041); the schedule equalizes only levied nickels</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>Bonds a nickel supports before state FSPK equalization</t>
-        </is>
-      </c>
-      <c r="B67" s="9">
-        <f>B66*(1-(1+B40)^-B41)/B40</f>
-        <v/>
+          <t>New annual state equalization on the recallable nickel (began FY2026)</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="n">
+        <v>276246</v>
       </c>
       <c r="F67" s="21" t="inlineStr">
         <is>
-          <t>FSPK equalization adds state dollars on top; KDE's tables set the amount</t>
+          <t>FY2027 SEEK schedule; $55,515 partial in FY2026. New restricted revenue, no board action required</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
+          <t>Bonds the new equalization alone supports</t>
+        </is>
+      </c>
+      <c r="B68" s="9">
+        <f>B67*(1-(1+B40)^-B41)/B40</f>
+        <v/>
+      </c>
+      <c r="F68" s="21" t="inlineStr">
+        <is>
+          <t>Additive to the FY2024 audit's bonding potential, which predates the equalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
           <t>SFCC offers of assistance, typical cycle</t>
         </is>
       </c>
-      <c r="B68" s="8" t="n">
+      <c r="B69" s="8" t="n">
         <v>1750000</v>
       </c>
-      <c r="F68" s="21" t="inlineStr">
+      <c r="F69" s="21" t="inlineStr">
         <is>
           <t>State already pays $1,568,809 of current principal</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>FY2026 YEAR-END, DISTRICT'S OWN KDE BUDGET MONITORING TOOL (UNAUDITED)</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>June 2026 financial packet, board agenda July 16, 2026; MUNIS run July 15, 2026. Audit will finalize these figures.</t>
         </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>General Fund revenue, FY2026 actual (excludes carryforward and on-behalf)</t>
-        </is>
-      </c>
-      <c r="B72" s="8" t="n">
-        <v>22103877</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>General Fund expenditures, FY2026 actual</t>
+          <t>General Fund revenue, FY2026 actual (excludes carryforward and on-behalf)</t>
         </is>
       </c>
       <c r="B73" s="8" t="n">
-        <v>22477866</v>
+        <v>22103877</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>Net General Fund change, FY2026 (unaudited)</t>
-        </is>
-      </c>
-      <c r="B74" s="30">
-        <f>B72-B73</f>
-        <v/>
-      </c>
-      <c r="F74" s="21" t="inlineStr">
-        <is>
-          <t>Compare net changes of -$1,065,657 in FY2024 and -$1,225,465 in FY2025 (audited)</t>
-        </is>
+          <t>General Fund expenditures, FY2026 actual</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="n">
+        <v>22477866</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Revenues over budget per the monitoring tool</t>
-        </is>
-      </c>
-      <c r="B75" s="8" t="n">
-        <v>2225835</v>
+          <t>Net General Fund change, FY2026 (unaudited)</t>
+        </is>
+      </c>
+      <c r="B75" s="30">
+        <f>B73-B74</f>
+        <v/>
+      </c>
+      <c r="F75" s="21" t="inlineStr">
+        <is>
+          <t>Compare net changes of -$1,065,657 in FY2024 and -$1,225,465 in FY2025 (audited)</t>
+        </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>Salaries under budget per the monitoring tool</t>
+          <t>Revenues over budget per the monitoring tool</t>
         </is>
       </c>
       <c r="B76" s="8" t="n">
-        <v>587592</v>
+        <v>2225835</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Salaries below FY2025 actuals</t>
+          <t>Salaries under budget per the monitoring tool</t>
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>223974</v>
+        <v>587592</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
+          <t>Salaries below FY2025 actuals</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="n">
+        <v>223974</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
           <t>Caveat: miscellaneous revenue budgeted at zero, received</t>
         </is>
       </c>
-      <c r="B78" s="8" t="n">
+      <c r="B79" s="8" t="n">
         <v>1567829</v>
       </c>
-      <c r="F78" s="21" t="inlineStr">
+      <c r="F79" s="21" t="inlineStr">
         <is>
           <t>If one-time, the underlying gap is about $1.9 million; the district should identify this receipt</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
         <is>
           <t>SCENARIO: BALANCE THE BUDGET AND EXPAND BONDING CAPACITY, NO CLOSURE</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>Two cases differ only in the operating gap assumed. Conservative treats the FY2026 $1.57M receipt as one-time;</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
+          <t>Two cases differ only in the operating gap assumed. Conservative treats the FY2026 $1.57M receipt as one-time;</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
           <t>trend uses the unaudited FY2026 net change. Operations are balanced first; only the remainder services debt.</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="B83" s="17" t="inlineStr">
+    <row r="84">
+      <c r="B84" s="17" t="inlineStr">
         <is>
           <t>Conservative</t>
         </is>
       </c>
-      <c r="C83" s="17" t="inlineStr">
+      <c r="C84" s="17" t="inlineStr">
         <is>
           <t>FY2026 trend</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
-        <is>
-          <t>Operating gap to close first</t>
-        </is>
-      </c>
-      <c r="B84" s="8" t="n">
-        <v>1900000</v>
-      </c>
-      <c r="C84" s="8" t="n">
-        <v>373989</v>
-      </c>
-      <c r="F84" s="21" t="inlineStr">
-        <is>
-          <t>Editable. $1.9M = FY2026 result excluding the unidentified receipt; $373,989 = FY2026 unaudited net change</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>New recurring revenue: 4 percent levy taken three years running</t>
-        </is>
-      </c>
-      <c r="B85" s="18">
-        <f>Tax_History!B32*(1.04^3-1)</f>
-        <v/>
-      </c>
-      <c r="C85" s="18">
-        <f>Tax_History!B32*(1.04^3-1)</f>
-        <v/>
+          <t>Operating gap to close first</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="C85" s="8" t="n">
+        <v>373989</v>
       </c>
       <c r="F85" s="21" t="inlineStr">
         <is>
-          <t>Same base and compounding as the levy tab; year 1 is $313,162, year 3 cumulative $977,568</t>
+          <t>Editable. $1.9M = FY2026 result excluding the unidentified receipt; $373,989 = FY2026 unaudited net change</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>Recurring cost reductions, not from closing a school</t>
-        </is>
-      </c>
-      <c r="B86" s="8" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="C86" s="8" t="n">
-        <v>1000000</v>
+          <t>New recurring revenue: 4 percent levy taken three years running</t>
+        </is>
+      </c>
+      <c r="B86" s="18">
+        <f>Tax_History!B32*(1.04^3-1)</f>
+        <v/>
+      </c>
+      <c r="C86" s="18">
+        <f>Tax_History!B32*(1.04^3-1)</f>
+        <v/>
       </c>
       <c r="F86" s="21" t="inlineStr">
         <is>
-          <t>Editable. For scale from the FY2025 audit: district administration grew $221K in one year, salaries fell $224K through attrition, spending ran $859K under budget</t>
+          <t>Same base and compounding as the levy tab; year 1 is $313,162, year 3 cumulative $977,568</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Operating room left for debt service after the budget balances</t>
-        </is>
-      </c>
-      <c r="B87" s="9">
-        <f>MAX(0,B85+B86-B84)</f>
-        <v/>
-      </c>
-      <c r="C87" s="9">
-        <f>MAX(0,C85+C86-C84)</f>
-        <v/>
+          <t>Recurring cost reductions, not from closing a school</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="C87" s="8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="F87" s="21" t="inlineStr">
+        <is>
+          <t>Editable. For scale from the FY2025 audit: district administration grew $221K in one year, salaries fell $224K through attrition, spending ran $859K under budget</t>
+        </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>General-fund bond capacity from that room</t>
+          <t>Operating room left for debt service after the budget balances</t>
         </is>
       </c>
       <c r="B88" s="9">
-        <f>B87*(1-(1+B$40)^-B$41)/B$40</f>
+        <f>MAX(0,B86+B87-B85)</f>
         <v/>
       </c>
       <c r="C88" s="9">
-        <f>C87*(1-(1+B$40)^-B$41)/B$40</f>
+        <f>MAX(0,C86+C87-C85)</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>Recallable nickel yield, restricted, before FSPK equalization</t>
+          <t>General-fund bond capacity from that room</t>
         </is>
       </c>
       <c r="B89" s="9">
-        <f>B65*0.0005</f>
+        <f>B88*(1-(1+B$40)^-B$41)/B$40</f>
         <v/>
       </c>
       <c r="C89" s="9">
-        <f>B65*0.0005</f>
+        <f>C88*(1-(1+B$40)^-B$41)/B$40</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Bond capacity from the nickel</t>
-        </is>
-      </c>
-      <c r="B90" s="9">
-        <f>B89*(1-(1+B$40)^-B$41)/B$40</f>
-        <v/>
-      </c>
-      <c r="C90" s="9">
-        <f>C89*(1-(1+B$40)^-B$41)/B$40</f>
-        <v/>
+          <t>New state equalization on the already-levied recallable nickel</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="n">
+        <v>276246</v>
+      </c>
+      <c r="C90" s="8" t="n">
+        <v>276246</v>
+      </c>
+      <c r="F90" s="21" t="inlineStr">
+        <is>
+          <t>FY2027 SEEK schedule; the recallable nickel itself is already levied and its local yield is already inside the building-fund stream above</t>
+        </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
+          <t>Bond capacity from the new equalization</t>
+        </is>
+      </c>
+      <c r="B91" s="9">
+        <f>B90*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+      <c r="C91" s="9">
+        <f>C90*(1-(1+B$40)^-B$41)/B$40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
           <t>Existing unused restricted capacity, approximate</t>
         </is>
       </c>
-      <c r="B91" s="8" t="n">
+      <c r="B92" s="8" t="n">
         <v>17600000</v>
       </c>
-      <c r="C91" s="8" t="n">
+      <c r="C92" s="8" t="n">
         <v>17600000</v>
       </c>
-      <c r="F91" s="21" t="inlineStr">
+      <c r="F92" s="21" t="inlineStr">
         <is>
           <t>FY2024 audit $23.5M less local share of the 2024 issue; fiscal agent's statement is the authority</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="22" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="22" t="inlineStr">
         <is>
           <t>Total capacity available without closing a school</t>
         </is>
       </c>
-      <c r="B92" s="24">
-        <f>B88+B90+B91</f>
-        <v/>
-      </c>
-      <c r="C92" s="24">
-        <f>C88+C90+C91</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>Roughly $30.6 million in the conservative case and $50.4 million on the FY2026 trend, with the budget balanced</t>
-        </is>
+      <c r="B93" s="24">
+        <f>B89+B91+B92</f>
+        <v/>
+      </c>
+      <c r="C93" s="24">
+        <f>C89+C91+C92</f>
+        <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Roughly $22.2 million in the conservative case and $42.1 million on the FY2026 trend, with the budget balanced</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>first in both. The administration's plan reaches $32 million at face value and leaves the deficit in place.</t>
         </is>

</xml_diff>

<commit_message>
Model: filled-to-capacity per-pupil comparison vs receiving schools
Redistricting tab: NMES per-pupil at 174 (state rating) and 154 (draft
rating), with and without added teachers, against Bourbon Central
($18,131) and Cane Ridge ($18,670) from the district's KDE 2023-24
filings. At capacity NMES becomes the cheapest elementary in the
district (~$14,300-$16,700 per pupil). 220 formulas; all tests green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -6070,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -6453,6 +6453,125 @@
       <c r="A43" s="21" t="inlineStr">
         <is>
           <t>Per-student figures pair the latest published spending year (2023-24) with the current enrollment count; refresh when the 2024-25 spending data posts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>FILLED-TO-CAPACITY PER-PUPIL COST VS THE RECEIVING SCHOOLS (KDE 2023-24 filings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Bourbon Central per pupil today</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="n">
+        <v>18131</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>District's own KDE school-level filing, 2023-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Cane Ridge per pupil today</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="n">
+        <v>18670</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Same filing; Cane Ridge runs 31 students over its rated capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>NMES per pupil today</t>
+        </is>
+      </c>
+      <c r="B48" s="18">
+        <f>Assumptions!B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>NMES filled to 174 (state-approved rating), no added teachers</t>
+        </is>
+      </c>
+      <c r="B49" s="9">
+        <f>(B34+(B6-B5)*Assumptions!B62)/B6</f>
+        <v/>
+      </c>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>Nine existing homerooms average 19.3 students at 174, inside every KRS 157.360 cap; only variable costs added</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>NMES filled to 174, conservative (two teachers added anyway)</t>
+        </is>
+      </c>
+      <c r="B50" s="9">
+        <f>(B34+2*Assumptions!B41+(B6-B5)*Assumptions!B62)/B6</f>
+        <v/>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>Adds two loaded certified positions even though class sizes do not require them</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>NMES filled to 154 (2026 draft plan rating), no added teachers</t>
+        </is>
+      </c>
+      <c r="B51" s="9">
+        <f>(B34+(154-B5)*Assumptions!B62)/154</f>
+        <v/>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>Same math at the draft plan's lower rating; class sizes average 17.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="inlineStr">
+        <is>
+          <t>NMES at 174 vs cheapest receiving school</t>
+        </is>
+      </c>
+      <c r="B52" s="24">
+        <f>B49-MIN(B46,B47)</f>
+        <v/>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>Negative = NMES becomes the cheapest elementary school in the district</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="21" t="inlineStr">
+        <is>
+          <t>Filling the school reverses the cost argument: the premium exists because fixed costs sit on 128 students; spread over 174 the same school costs less per child than either receiving school, and the transfer students free the exact seats Cane Ridge is over capacity by.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Model: sensitivity analysis on the filled-to-capacity per-pupil result
Redistricting tab: break-even marginal cost per added student at both
capacity ratings vs both receiving schools (14.7K/16.8K at 174;
12.1K/15.3K at 154), a per-pupil grid across marginal-cost assumptions
(400 to the full 14,173 state/local average), and base-year variant at
115 enrolled. Verdict: structural at the state-approved 174 rating,
robust at the draft 154 rating. 235 formulas; all tests green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -6070,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -6572,6 +6572,188 @@
       <c r="A53" s="21" t="inlineStr">
         <is>
           <t>Filling the school reverses the cost argument: the premium exists because fixed costs sit on 128 students; spread over 174 the same school costs less per child than either receiving school, and the transfer students free the exact seats Cane Ridge is over capacity by.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>SENSITIVITY: IS THE CAPACITY RESULT STRUCTURAL, OR AN ARTIFACT OF ASSUMPTIONS?</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="inlineStr">
+        <is>
+          <t>The only lever that matters is the marginal cost of each added student. Break-even values below are the marginal cost at which NMES at capacity stops being cheaper. Compare them to reality: added supplies and materials run a few hundred dollars; even hiring staff in proportion to students costs roughly half the average, because the average includes the principal, building, and staff already paid for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Break-even marginal cost, NMES at 174 vs Bourbon Central</t>
+        </is>
+      </c>
+      <c r="B57" s="9">
+        <f>(B46*B6-B34)/(B6-B5)</f>
+        <v/>
+      </c>
+      <c r="C57" s="21" t="inlineStr">
+        <is>
+          <t>NMES stays cheaper than Bourbon Central for any marginal cost below this</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Break-even marginal cost, NMES at 174 vs Cane Ridge</t>
+        </is>
+      </c>
+      <c r="B58" s="9">
+        <f>(B47*B6-B34)/(B6-B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Break-even marginal cost, NMES at 154 vs Bourbon Central</t>
+        </is>
+      </c>
+      <c r="B59" s="9">
+        <f>(B46*154-B34)/(154-B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Break-even marginal cost, NMES at 154 vs Cane Ridge</t>
+        </is>
+      </c>
+      <c r="B60" s="9">
+        <f>(B47*154-B34)/(154-B5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Reference: NMES's ENTIRE state and local spending per pupil (fixed costs included)</t>
+        </is>
+      </c>
+      <c r="B61" s="18">
+        <f>Assumptions!B15</f>
+        <v/>
+      </c>
+      <c r="C61" s="21" t="inlineStr">
+        <is>
+          <t>Even if every added student cost this full amount, which is impossible since it includes the fixed costs already paid, NMES at 174 still comes in under both receiving schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>PER-PUPIL GRID ACROSS MARGINAL-COST ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Marginal cost per added student</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="inlineStr">
+        <is>
+          <t>At 174</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>At 154</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="B65" s="9">
+        <f>(B$34+(B$6-B$5)*A65)/B$6</f>
+        <v/>
+      </c>
+      <c r="C65" s="9">
+        <f>(B$34+(154-B$5)*A65)/154</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="B66" s="9">
+        <f>(B$34+(B$6-B$5)*A66)/B$6</f>
+        <v/>
+      </c>
+      <c r="C66" s="9">
+        <f>(B$34+(154-B$5)*A66)/154</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B67" s="9">
+        <f>(B$34+(B$6-B$5)*A67)/B$6</f>
+        <v/>
+      </c>
+      <c r="C67" s="9">
+        <f>(B$34+(154-B$5)*A67)/154</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B68" s="9">
+        <f>(B$34+(B$6-B$5)*A68)/B$6</f>
+        <v/>
+      </c>
+      <c r="C68" s="9">
+        <f>(B$34+(154-B$5)*A68)/154</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n">
+        <v>14173</v>
+      </c>
+      <c r="B69" s="9">
+        <f>(B$34+(B$6-B$5)*A69)/B$6</f>
+        <v/>
+      </c>
+      <c r="C69" s="9">
+        <f>(B$34+(154-B$5)*A69)/154</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="21" t="inlineStr">
+        <is>
+          <t>Receiving schools today: Bourbon Central $18,131, Cane Ridge $18,670. At the state-approved 174 rating, NMES undercuts both across the entire grid, including the impossible full-average case. At the draft plan's 154 rating it holds for any marginal cost under about $12,000, roughly thirty times the realistic figure. Verdict: structural at 174, robust at 154.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="21" t="inlineStr">
+        <is>
+          <t>Base-year variant: at the current 115 enrolled, filling to 174 adds 59 students and the break-even vs Bourbon Central falls to about $11,500, with the same verdict. Two added teachers at the loaded rate are equivalent to about $3,700 of marginal cost per student, inside the grid above.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Figure 6 + site chart: per-pupil across schools over time with capacity counterfactual
- New chart (site Chart.js + report Figure 6): actual per-pupil for NMES,
  Bourbon Central, Cane Ridge across all five KDE filing years (2019-20
  to 2023-24), with a dashed NMES-filled-to-174 counterfactual that sits
  below both receiving schools in every year
- Report Section 4: new figure and paragraph; spending growth comparison
  (NMES +16% vs BCES +37% / CRES +47%); figures 6-15 renumbered to 7-16
  with cross-references updated in model and sync check
- Site: new card after Room to grow with the chart and stress-test text
- Model Redistricting tab: five-year table backing the figure
  (240 formulas); README counts refreshed; report now 36 pages
- Tests: site expects 7 charts; new checks pin Figure 6 and key values

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -656,21 +656,21 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  County demographics and the full 1989-2025 NMES enrollment series: Demographics tab (backs Section 9 and Figure 11).</t>
+          <t xml:space="preserve">  County demographics and the full 1989-2025 NMES enrollment series: Demographics tab (backs Section 9 and Figure 12).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tax rates, fund split, delinquency check, and the 4% three-year path: Tax_History tab (backs Figure 15).</t>
+          <t xml:space="preserve">  Tax rates, fund split, delinquency check, and the 4% three-year path: Tax_History tab (backs Figure 16).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Boundary rebalancing and fill-to-capacity scenario: Redistricting tab (backs the Section 9 worked example and Figure 12).</t>
+          <t xml:space="preserve">  Boundary rebalancing and fill-to-capacity scenario: Redistricting tab (backs the Section 9 worked example and Figure 13).</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Backs Section 9 and Figure 15 of the report. Rates in cents per $100. DOR rate books primary for 2023-2025; 2018-2022 verified secondary; 2005-2017 not retrieved and not interpolated.</t>
+          <t>Backs Section 9 and Figure 16 of the report. Rates in cents per $100. DOR rate books primary for 2023-2025; 2018-2022 verified secondary; 2005-2017 not retrieved and not interpolated.</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>NMES ENROLLMENT, 1989-2025 (spring of school year; backs Figure 11)</t>
+          <t>NMES ENROLLMENT, 1989-2025 (spring of school year; backs Figure 12)</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>NMES ENROLLMENT BY SCHOOL YEAR (backs Figure 11)</t>
+          <t>NMES ENROLLMENT BY SCHOOL YEAR (backs Figure 12)</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -6754,6 +6754,167 @@
       <c r="A71" s="21" t="inlineStr">
         <is>
           <t>Base-year variant: at the current 115 enrolled, filling to 174 adds 59 students and the break-even vs Bourbon Central falls to about $11,500, with the same verdict. Two added teachers at the loaded rate are equivalent to about $3,700 of marginal cost per student, inside the grid above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>FIVE YEARS OF THE SAME TEST (KDE school-level filings, 2019-20 to 2023-24; backs Figure 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>NMES members</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="inlineStr">
+        <is>
+          <t>NMES $/pupil</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="inlineStr">
+        <is>
+          <t>BCES $/pupil</t>
+        </is>
+      </c>
+      <c r="E74" s="17" t="inlineStr">
+        <is>
+          <t>CRES $/pupil</t>
+        </is>
+      </c>
+      <c r="F74" s="17" t="inlineStr">
+        <is>
+          <t>NMES at 174</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2019-20</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="n">
+        <v>166</v>
+      </c>
+      <c r="C75" s="8" t="n">
+        <v>12903</v>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>12159</v>
+      </c>
+      <c r="E75" s="8" t="n">
+        <v>12168</v>
+      </c>
+      <c r="F75" s="9">
+        <f>(C75*B75+(174-B75)*Assumptions!B62)/174</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2020-21</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="n">
+        <v>160</v>
+      </c>
+      <c r="C76" s="8" t="n">
+        <v>15406</v>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>14011</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>14621</v>
+      </c>
+      <c r="F76" s="9">
+        <f>(C76*B76+(174-B76)*Assumptions!B62)/174</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2021-22</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="n">
+        <v>146</v>
+      </c>
+      <c r="C77" s="8" t="n">
+        <v>19080</v>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>15619</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>16137</v>
+      </c>
+      <c r="F77" s="9">
+        <f>(C77*B77+(174-B77)*Assumptions!B62)/174</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>2022-23</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="n">
+        <v>144</v>
+      </c>
+      <c r="C78" s="8" t="n">
+        <v>19003</v>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>17410</v>
+      </c>
+      <c r="E78" s="8" t="n">
+        <v>17403</v>
+      </c>
+      <c r="F78" s="9">
+        <f>(C78*B78+(174-B78)*Assumptions!B62)/174</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>2023-24</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="n">
+        <v>128</v>
+      </c>
+      <c r="C79" s="8" t="n">
+        <v>19348</v>
+      </c>
+      <c r="D79" s="8" t="n">
+        <v>18131</v>
+      </c>
+      <c r="E79" s="8" t="n">
+        <v>18670</v>
+      </c>
+      <c r="F79" s="9">
+        <f>(C79*B79+(174-B79)*Assumptions!B62)/174</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="21" t="inlineStr">
+        <is>
+          <t>The counterfactual column is below both receiving schools in every year on record. NMES's total site spending grew 16 percent over the five years, against 37 percent at Bourbon Central and 47 percent at Cane Ridge; only the divisor changed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Symmetry check: sender-side per-pupil effect of filling NMES
Apply the denominator effect both ways: sending students out of Bourbon
Central and Cane Ridge raises their per-pupil to roughly $18,700/$19,300
(scenario) or $19,000/$19,600 (all-in-county stress), since departing
students take only variable cost. Model Redistricting tab adds the
post-move comparison (244 formulas); site card and report Section 4 add
the honest caution: per-pupil is a utilization measure, a shuffle is
cost-neutral district-wide, NMES at 174 stays cheapest by a wider margin
after the move, and the same symmetry undercuts the closure's optics.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -6070,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -6915,6 +6915,81 @@
       <c r="A81" s="21" t="inlineStr">
         <is>
           <t>The counterfactual column is below both receiving schools in every year on record. NMES's total site spending grew 16 percent over the five years, against 37 percent at Bourbon Central and 47 percent at Cane Ridge; only the divisor changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>SYMMETRY CHECK: THE SENDERS' PER-PUPIL AFTER THE MOVE (2023-24 basis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="21" t="inlineStr">
+        <is>
+          <t>Per-pupil rises at the senders for the same denominator reason it falls at NMES; a pure shuffle leaves total district spending nearly unchanged in either direction. The comparison below is the honest post-move one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Bourbon Central after sending 15 rezoned students</t>
+        </is>
+      </c>
+      <c r="B85" s="9">
+        <f>(8902321-15*Assumptions!B62)/(491-15)</f>
+        <v/>
+      </c>
+      <c r="C85" s="21" t="inlineStr">
+        <is>
+          <t>2023-24 filing: $8,902,321 across 491 members; loses only variable cost per departing student</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Cane Ridge after sending 15 rezoned students</t>
+        </is>
+      </c>
+      <c r="B86" s="9">
+        <f>(8606870-15*Assumptions!B62)/(461-15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Stress case: all 46 drawn in-county, 23 from each sender</t>
+        </is>
+      </c>
+      <c r="B87" s="9">
+        <f>(8902321-23*Assumptions!B62)/(491-23)</f>
+        <v/>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Bourbon Central; Cane Ridge in the next row</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Stress case, Cane Ridge</t>
+        </is>
+      </c>
+      <c r="B88" s="9">
+        <f>(8606870-23*Assumptions!B62)/(461-23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="21" t="inlineStr">
+        <is>
+          <t>NMES at 174 stays the cheapest of the three after the move, by a wider margin than before it (about $4,400 vs $3,800). The district-level cash case is booked separately and conservatively above as the net recurring benefit: consolidated sections at the senders, HB 563 SEEK revenue from out-of-county transfers, and capacity relief at Cane Ridge, which runs 31 students over its rating. The same symmetry runs the other way: closing NMES would lower the receiving schools' per-pupil optics while saving almost nothing in total, which is the closure case's weakness in one sentence.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct Figure 6 overclaim; validate capacity result at both ratings over time
Self-caught correction: the filled-to-174 counterfactual was within 1-3
percent ABOVE the cheapest school in 2019-22 (a tie, not cheapest), and
is decisively cheapest only in 2022-23 and 2023-24. Figure 6, the site
card, and the model note now say so plainly. The single figure now
carries both counterfactuals: filled to 174 (approved rating) and filled
to 154 (draft plan's proposed rating, plotted from 2021-22 because the
school enrolled 166 and 160 before that, above the proposed rating).
In current costs the filled school is cheapest at BOTH ratings ($14,339
and $16,149 vs $18,131/$18,670). Model adds the at-154 column (247
formulas); report now 37 pages; new tests pin the corrected wording.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -6070,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -6795,6 +6795,11 @@
           <t>NMES at 174</t>
         </is>
       </c>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>NMES at 154</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -6818,6 +6823,11 @@
         <f>(C75*B75+(174-B75)*Assumptions!B62)/174</f>
         <v/>
       </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>n/a: enrolled above 154</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -6841,6 +6851,11 @@
         <f>(C76*B76+(174-B76)*Assumptions!B62)/174</f>
         <v/>
       </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>n/a: enrolled above 154</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -6864,6 +6879,10 @@
         <f>(C77*B77+(174-B77)*Assumptions!B62)/174</f>
         <v/>
       </c>
+      <c r="G77" s="9">
+        <f>(C77*B77+(154-B77)*Assumptions!B62)/154</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -6887,6 +6906,10 @@
         <f>(C78*B78+(174-B78)*Assumptions!B62)/174</f>
         <v/>
       </c>
+      <c r="G78" s="9">
+        <f>(C78*B78+(154-B78)*Assumptions!B62)/154</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -6910,11 +6933,15 @@
         <f>(C79*B79+(174-B79)*Assumptions!B62)/174</f>
         <v/>
       </c>
+      <c r="G79" s="9">
+        <f>(C79*B79+(154-B79)*Assumptions!B62)/154</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="21" t="inlineStr">
         <is>
-          <t>The counterfactual column is below both receiving schools in every year on record. NMES's total site spending grew 16 percent over the five years, against 37 percent at Bourbon Central and 47 percent at Cane Ridge; only the divisor changed.</t>
+          <t>Honest reading (corrected 7/26): at 174 the counterfactual is within 1 to 3 percent of the cheapest school in 2019-22, a tie, and decisively below both schools in 2022-23 and 2023-24. At the draft plan's 154 rating it is cheapest on the 2023-24 filing; in 2019-20 and 2020-21 the school enrolled above 154, the capacity the draft now assigns it. NMES's total site spending grew 16 percent over the five years, against 37 percent at Bourbon Central and 47 percent at Cane Ridge; only the divisor changed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Variable-cost validation for the capacity scenario, both directions
Price staffing instead of assuming it away: KRS 157.360 class caps at an
even grade mix require ~11 sections at 174 and ~10 at 154 against 9
existing rooms, so the staffed cases ($15,316 at 174 with two added
teachers, $16,701 at 154 with one) are the honest base cases; both stay
cheapest of the three schools in current costs. Long-run bound (every
added student at the full $14,173 S/L average) holds at 174 ($17,980),
fails at 154 as the break-even rows already showed. Sender-side check
with a consolidated section each: $18,511/$19,094, still ~$3,000 above
the staffed NMES cases, with a no-double-counting note. Same discipline
stated for the closure direction. Site card and Figure 6 caption updated;
model adds the validation block (252 formulas); tests pin the staffed
figures.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -6070,7 +6070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -7017,6 +7017,97 @@
       <c r="A89" s="21" t="inlineStr">
         <is>
           <t>NMES at 174 stays the cheapest of the three after the move, by a wider margin than before it (about $4,400 vs $3,800). The district-level cash case is booked separately and conservatively above as the net recurring benefit: consolidated sections at the senders, HB 563 SEEK revenue from out-of-county transfers, and capacity relief at Cane Ridge, which runs 31 students over its rating. The same symmetry runs the other way: closing NMES would lower the receiving schools' per-pupil optics while saving almost nothing in total, which is the closure case's weakness in one sentence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>VARIABLE-COST VALIDATION, BOTH DIRECTIONS (added 7/26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="21" t="inlineStr">
+        <is>
+          <t>Class-cap staffing check (KRS 157.360: 24 in K-3, 28 in grade 4, 29 in grade 5). At an even grade mix, 174 students need about 11 sections against 9 existing rooms, and 154 need about 10; the supplies-only counterfactual is therefore the BEST case, and the staffed cases below are the honest base cases. Grade-by-grade enrollment is a records ask; a mix weighted to grades 4-5 needs fewer sections.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>NMES at 174 with two added sections (base case)</t>
+        </is>
+      </c>
+      <c r="B93" s="9">
+        <f>(B34+2*Assumptions!B41+(B6-B5)*Assumptions!B62)/B6</f>
+        <v/>
+      </c>
+      <c r="C93" s="21" t="inlineStr">
+        <is>
+          <t>Same as the conservative row above; cheapest of the three on the 2023-24 filing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>NMES at 154 with one added section (base case)</t>
+        </is>
+      </c>
+      <c r="B94" s="9">
+        <f>(B34+Assumptions!B41+(154-B5)*Assumptions!B62)/154</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>Long-run bound at 174: every added student at the full $14,173 S/L average</t>
+        </is>
+      </c>
+      <c r="B95" s="9">
+        <f>(B34+(B6-B5)*Assumptions!B15)/B6</f>
+        <v/>
+      </c>
+      <c r="C95" s="21" t="inlineStr">
+        <is>
+          <t>Still under both receiving schools on the 2023-24 filing. At 154 the same bound gives $18,474 and fails against Bourbon Central, consistent with the break-even rows above</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Senders after 15 out each WITH one consolidated section (favorable to senders)</t>
+        </is>
+      </c>
+      <c r="B96" s="9">
+        <f>(8902321-15*Assumptions!B62-Assumptions!B41)/(491-15)</f>
+        <v/>
+      </c>
+      <c r="C96" s="21" t="inlineStr">
+        <is>
+          <t>Bourbon Central; Cane Ridge next row. Consolidation lowers sender per-pupil AND is the source of the district-level saving; do not count it twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Cane Ridge, same treatment</t>
+        </is>
+      </c>
+      <c r="B97" s="9">
+        <f>(8606870-15*Assumptions!B62-Assumptions!B41)/(461-15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net saving is $121K to $725K and not the school's $2.5M gross cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix three-plans table: closure runway recomputed on v3 economics
The Reserves-in-2029 column and footnote still used the retired $361K
base case (via the old $85K position cost feeding Runway). Now: closure
path runs on the v3 central case ($131,240); at the median the reserves
are gone on nearly the status-quo schedule (FY2029 about -$18K), central
case about $0.1M, best case $1.4M; site, PDF Section 12 table/caption,
Closure_Model base block (GF-borne positions), and Runway tab all agree;
v3.0 archive copy refreshed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -823,7 +823,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Closure only (base-case net saving from FY2027)</t>
+          <t>Closure only (v3 central case, $131,240, from FY2027)</t>
         </is>
       </c>
       <c r="B7" s="9">
@@ -831,15 +831,15 @@
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>B7-GF_Summary!$D$16+Closure_Model!$B$20</f>
+        <f>B7-GF_Summary!$D$16+Closure_Model!$B$47</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>C7-GF_Summary!$D$16+Closure_Model!$B$20</f>
+        <f>C7-GF_Summary!$D$16+Closure_Model!$B$47</f>
         <v/>
       </c>
       <c r="E7" s="9">
-        <f>D7-GF_Summary!$D$16+Closure_Model!$B$20</f>
+        <f>D7-GF_Summary!$D$16+Closure_Model!$B$47</f>
         <v/>
       </c>
     </row>
@@ -864,6 +864,13 @@
       <c r="E8" s="18">
         <f>GF_Summary!$D$14</f>
         <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Closure range check (v3): at the +$565,000 best case FY2029 ends near $1.4M; at the +$91,240 median the reserves are gone on nearly the status-quo schedule; in the 29 percent of scenarios that lose money, sooner than status quo.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -5774,12 +5781,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Teaching positions eliminated (via attrition)</t>
+          <t>Teaching positions eliminated (via attrition, GF-borne cost)</t>
         </is>
       </c>
       <c r="B12" s="18">
-        <f>Assumptions!B53*Assumptions!B41</f>
-        <v/>
+        <f>Assumptions!B53*Assumptions!B69</f>
+        <v/>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>v3: GF-borne $60K per position (state pays TRS/KEHP on-behalf); prior versions used the $85K all-in figure here</t>
+        </is>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Cite provenance: built from public records and Open Records Requests only
The provenance line now appears on the site (top disclosure and footer),
the report (title page, scope box, and notes on the data), the executive
summary header, and the model's read-me caveat. The scope box also names
KRS 61.870 as the basis for the district-produced documents. Validation
now enforces the phrase on both the site and the report.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -720,14 +720,21 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Prepared by a former NMES King working alongside Claude, an AI research assistant from Anthropic. Estimates are labeled; every figure</t>
+          <t>Prepared by a former NMES King working alongside Claude, an AI research assistant from Anthropic. Built from public records and</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>should be re-verified against the cited primary sources before formal use. Nothing here alleges misconduct by any official.</t>
+          <t>Open Records Requests only. Estimates are labeled; every figure should be re-verified against the cited primary sources before</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>formal use. Nothing here alleges misconduct by any official.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove shared services with Paris Independent from the cost menu
The lever-2 list is now four items, worth $760,000 to $1.3 million a
year counted once (was five at $860,000 to $1.6 million). Downstream
renumbering: raw menu $1.4 to $2.3 million, published conservative
band $0.9 to $1.7 million (midpoint $1.3 million into the Runway
sheet, with the Alternatives reference re-pinned after the row shift),
plan-3 FY2029 balance about $2.9 million, and the plan's low-end sum
about $1.9 million a year covering about 70 percent of the gap. Sync
recomputes every band from the raw rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -834,15 +834,15 @@
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>B6-GF_Summary!$D$16+0.5*Alternatives!$B$20</f>
+        <f>B6-GF_Summary!$D$16+0.5*Alternatives!$B$19</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>C6-GF_Summary!$D$16+Alternatives!$B$20</f>
+        <f>C6-GF_Summary!$D$16+Alternatives!$B$19</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>D6-GF_Summary!$D$16+Alternatives!$B$20</f>
+        <f>D6-GF_Summary!$D$16+Alternatives!$B$19</f>
         <v/>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B7" s="18">
-        <f>Alternatives!B20</f>
+        <f>Alternatives!B19</f>
         <v/>
       </c>
       <c r="C7" s="9">
@@ -12054,7 +12054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -12315,253 +12315,225 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Shared services with Paris Independent</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>300000</v>
+          <t>Fill NMES to capacity (rebalance + transfers, net)</t>
+        </is>
+      </c>
+      <c r="B11" s="18">
+        <f>Redistricting!B30</f>
+        <v/>
+      </c>
+      <c r="C11" s="18">
+        <f>Redistricting!B31</f>
+        <v/>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Transport, food service, back office</t>
+          <t>Boundary rebalancing and cross-county scenario, Redistricting tab</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Cost reduction</t>
+          <t>New revenue, net of costs</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Low; needs an interlocal feasibility study</t>
+          <t>High; board boundary authority, math on Redistricting tab</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Fill NMES to capacity (rebalance + transfers, net)</t>
+          <t>District-wide recruitment beyond NMES's 46 seats (homeschool, private-school, nonresident incentives; v3.8)</t>
         </is>
       </c>
       <c r="B12" s="18">
-        <f>Redistricting!B30</f>
+        <f>25*(Assumptions!B6-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="C12" s="18">
-        <f>Redistricting!B31</f>
+        <f>50*(Assumptions!B6-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Boundary rebalancing and cross-county scenario, Redistricting tab</t>
+          <t>25-50 additional students at $4,226 net; pool measured on Redistricting rows 116-135 (259 registered homeschoolers, ACS pool ~1,135, net import already 189); 62 open seats exist at Bourbon Central's approved rating</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>New revenue, net of costs</t>
+          <t>New revenue</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>High; board boundary authority, math on Redistricting tab</t>
+          <t>Medium; needs an enrollment marketing plan and incentive design</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>District-wide recruitment beyond NMES's 46 seats (homeschool, private-school, nonresident incentives; v3.8)</t>
-        </is>
-      </c>
-      <c r="B13" s="18">
-        <f>25*(Assumptions!B6-Assumptions!B62)</f>
-        <v/>
-      </c>
-      <c r="C13" s="18">
-        <f>50*(Assumptions!B6-Assumptions!B62)</f>
-        <v/>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>25-50 additional students at $4,226 net; pool measured on Redistricting rows 116-135 (259 registered homeschoolers, ACS pool ~1,135, net import already 189); 62 open seats exist at Bourbon Central's approved rating</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>New revenue</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Medium; needs an enrollment marketing plan and incentive design</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Total identified (ranges overlap; not additive to the penny)</t>
         </is>
       </c>
-      <c r="B14" s="24">
-        <f>SUM(B4:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="24">
-        <f>SUM(C4:C13)</f>
-        <v/>
+      <c r="B13" s="24">
+        <f>SUM(B4:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="24">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>COMPARISON</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>COMPARISON</t>
-        </is>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Package midpoint (raw sum of ranges)</t>
+        </is>
+      </c>
+      <c r="B16" s="9">
+        <f>(B13+C13)/2</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Package midpoint (raw sum of ranges)</t>
-        </is>
-      </c>
-      <c r="B17" s="9">
-        <f>(B14+C14)/2</f>
-        <v/>
+          <t>Conservative combined estimate, low (haircut for overlap)</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="n">
+        <v>900000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Conservative combined estimate, low (haircut for overlap)</t>
+          <t>Conservative combined estimate, high</t>
         </is>
       </c>
       <c r="B18" s="14" t="n">
-        <v>1000000</v>
+        <v>1700000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Conservative combined estimate, high</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="n">
-        <v>1900000</v>
+          <t>Conservative midpoint (used in Runway sheet)</t>
+        </is>
+      </c>
+      <c r="B19" s="9">
+        <f>(B17+B18)/2</f>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Conservative midpoint (used in Runway sheet)</t>
-        </is>
-      </c>
-      <c r="B20" s="9">
-        <f>(B18+B19)/2</f>
+          <t>Average annual GF drawdown (FY2024-25)</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>GF_Summary!D16</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Average annual GF drawdown (FY2024-25)</t>
+          <t>Closure net saving (base case)</t>
         </is>
       </c>
       <c r="B21" s="18">
-        <f>GF_Summary!D16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Closure net saving (base case)</t>
-        </is>
-      </c>
-      <c r="B22" s="18">
         <f>Closure_Model!B20</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>Reading: raw row sums run about $1.5M to $2.6M; the published $1.0M to $1.9M band applies a conservative haircut for overlap and implementation risk. Medicaid and reimbursement recovery were removed from the menu in v4.2 review. Coverage is reported against both yardsticks: the $2.65M structural gap before transfers and the roughly $1.15M net drawdown after transfers (Closure_Model rows 21 and 35 carry both for closure).</t>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Reading: raw row sums run about $1.4M to $2.3M; the published $0.9M to $1.7M band applies a conservative haircut for overlap and implementation risk. Medicaid and reimbursement recovery were removed from the menu in v4.2 review; shared services with Paris Independent was removed in v4.4 review. Coverage is reported against both yardsticks: the $2.65M structural gap before transfers and the roughly $1.15M net drawdown after transfers (Closure_Model rows 21 and 35 carry both for closure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>THE GROWTH PATH: THE SAME MENU AS A DISTRICT-WIDE RECOVERY PLAN (v3.8; backs the site card and Section 9)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>THE GROWTH PATH: THE SAME MENU AS A DISTRICT-WIDE RECOVERY PLAN (v3.8; backs the site card and Section 9)</t>
-        </is>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Move 1: inspect fixed costs (every non-teaching position via attrition, administrative restructuring, transport, energy)</t>
+        </is>
+      </c>
+      <c r="B26" s="23">
+        <f>SUM(B7:B10)</f>
+        <v/>
+      </c>
+      <c r="C26" s="23">
+        <f>SUM(C7:C10)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Move 1: inspect fixed costs (every non-teaching position via attrition, administrative restructuring, transport, energy, shared services)</t>
+          <t>Move 2: grow enrollment instead of shrinking it (attendance recovery, fill NMES, district-wide recruitment)</t>
         </is>
       </c>
       <c r="B27" s="23">
-        <f>SUM(B7:B11)</f>
+        <f>B6+B11+B12</f>
         <v/>
       </c>
       <c r="C27" s="23">
-        <f>SUM(C7:C11)</f>
+        <f>C6+C11+C12</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Move 2: grow enrollment instead of shrinking it (attendance recovery, fill NMES, district-wide recruitment)</t>
+          <t>Move 3: the honest revenue conversation, year one (4 percent option plus delinquency; compounds by year three; recallable menu beyond it on Tax_History rows 70-91)</t>
         </is>
       </c>
       <c r="B28" s="23">
-        <f>B6+B12+B13</f>
+        <f>B4+B5</f>
         <v/>
       </c>
       <c r="C28" s="23">
-        <f>C6+C12+C13</f>
+        <f>C4+C5</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Move 3: the honest revenue conversation, year one (4 percent option plus delinquency; compounds by year three; recallable menu beyond it on Tax_History rows 70-91)</t>
+          <t>Growth plan total (equals the raw sum above; the published band is the conservative cut of the same rows)</t>
         </is>
       </c>
       <c r="B29" s="23">
-        <f>B4+B5</f>
+        <f>B26+B27+B28</f>
         <v/>
       </c>
       <c r="C29" s="23">
-        <f>C4+C5</f>
+        <f>C26+C27+C28</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>Growth plan total (equals the raw sum above; the published band is the conservative cut of the same rows)</t>
-        </is>
-      </c>
-      <c r="B30" s="23">
-        <f>B27+B28+B29</f>
-        <v/>
-      </c>
-      <c r="C30" s="23">
-        <f>C27+C28+C29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A30" s="21" t="inlineStr">
         <is>
           <t>NMES is not the reason salaries cannot rise (its honest excess cost is about $156,000, six tenths of a percent of the budget) and not the reason capital waits (about $17.6M of restricted capacity sits unused while the sweep drains the building fund). The structural problem is district-wide; so is the fix.</t>
         </is>

</xml_diff>

<commit_message>
Publish the menu band raw: $1.4 to $2.3 million, no haircut
The published band is now the raw row sums with no overlap haircut;
each line's confidence rating on the Alternatives tab carries the
uncertainty instead. Downstream: Runway midpoint rises to $1.87
million and the plan-3 FY2029 balance to about $4.3 million. Sync
pins the band to the recomputed row sums in both the model and the
report.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -12408,11 +12408,11 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Conservative combined estimate, low (haircut for overlap)</t>
+          <t>Published band, low (raw row sums, no haircut)</t>
         </is>
       </c>
       <c r="B17" s="14" t="n">
-        <v>900000</v>
+        <v>1393830</v>
       </c>
     </row>
     <row r="18">
@@ -12428,7 +12428,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Conservative midpoint (used in Runway sheet)</t>
+          <t>Band midpoint (used in Runway sheet)</t>
         </is>
       </c>
       <c r="B19" s="9">
@@ -12461,7 +12461,7 @@
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>Reading: raw row sums run about $1.4M to $2.3M; the published $0.9M to $1.7M band applies a conservative haircut for overlap and implementation risk. Medicaid and reimbursement recovery were removed from the menu in v4.2 review; shared services with Paris Independent was removed in v4.4 review. Coverage is reported against both yardsticks: the $2.65M structural gap before transfers and the roughly $1.15M net drawdown after transfers (Closure_Model rows 21 and 35 carry both for closure).</t>
+          <t>Reading: the published band IS the raw row sums, $1.4M to $2.3M, with no haircut (v4.4 review); ranges overlap and are not additive to the penny, and each line carries its own confidence rating in column F. Medicaid and reimbursement recovery were removed from the menu in v4.2 review; shared services with Paris Independent was removed in v4.4 review. Coverage is reported against both yardsticks: the $2.65M structural gap before transfers and the roughly $1.15M net drawdown after transfers (Closure_Model rows 21 and 35 carry both for closure).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan calculator opens at the central case: half the leakage pool recovered
The recovered-students slider now defaults to 275 of 550, worth
$1,162,150 a year at $4,226 each, so the default surplus is $1,882,976
over the trending fiscal 2026 gap: the 5 percent raise plus about
$17.9 million of new bonds, about $50 million of capacity with the
advisor's $32 million. The zero-recovery floor stays published beside it
($721,000 to spare, $2.8 million of bonds, about $35 million), the roads
panel mirrors the new default (+$3.6M of recurring resources), and the
report, model Alternatives tab, version history, and all three suites
carry the same chain.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -12542,11 +12542,11 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Plan levers at the website defaults: 0 leakage students recovered + costs at the $760K low end</t>
+          <t>Plan levers at the website defaults: 275 of 550 leakage students recovered (275 x $4,226 = $1,162,150) + costs at the $760K low end</t>
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>760000</v>
+        <v>1922150</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
@@ -12657,7 +12657,7 @@
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>Reading: at the website defaults (no recovery, costs at the low end, full restore) the plan clears the trending fiscal 2026 gap with about $721K to spare, funds the 5 percent certified raise, and still leaves about $214K for debt: about $2.8M of new GF-leveraged bonds plus the advisor's $32M, about $35 million of building capacity with every school open. Every 100 recovered leakage students add $422,600 a year on top; the website slider runs to the full 550. The earlier 10-percent-raise / $52M top-end claim is withdrawn with the lever correction.</t>
+          <t>Reading: at the website defaults (half the pool recovered, costs at the low end, full restore) the plan runs about $1.88M ahead of the trending fiscal 2026 gap, funds the 5 percent certified raise, and leaves about $1.38M for debt: about $17.9M of new GF-leveraged bonds plus the advisor's $32M, about $50 million of building capacity with every school open. The zero-recovery floor still clears the gap with about $721K to spare (raise + $2.8M of bonds, about $35M). Every 100 recovered leakage students move the surplus by $422,600 a year; the website slider runs 0 to 550. The earlier 10-percent-raise / $52M top-end claim is withdrawn with the lever correction.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price the leakage pool at the undiscounted SEEK base: $2.1 to $2.5 million
The 450 to 550 pool's headline pricing moves from the net-of-supplies
$4,226 cell to the full $4,626 SEEK base on all three artifacts, since
revenue the district is not collecting is the whole check: $2.1 to
$2.5 million a year. The net $1.9 to $2.3 million stays published in
Section 10 beside it, and the plan calculator still credits recovered
students only at $4,226. The model prices both bands as live formulas
(Redistricting rows 139 and 140), the version history discloses the
restatement, and validate recomputes both bands and pins the wording.
Also replaces a stale executive summary copy at the repo root (the
build script writes to the working directory, not /home/claude/nmes)
and removes the stray copy that briefly landed in build/.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -9928,7 +9928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56" customWidth="1" min="1" max="1"/>
@@ -11420,6 +11420,36 @@
         <is>
           <t>450 to 550</t>
         </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>Pool priced at the full SEEK base, revenue not collected today (450 and 550 x FY2027 base; the published $2.1 to $2.5 million)</t>
+        </is>
+      </c>
+      <c r="B139" s="23">
+        <f>450*Assumptions!B6</f>
+        <v/>
+      </c>
+      <c r="C139" s="23">
+        <f>550*Assumptions!B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>Same pool net of supplies, the basis the plan calculator credits per recovered student ($1.9 to $2.3 million)</t>
+        </is>
+      </c>
+      <c r="B140" s="9">
+        <f>450*(Assumptions!B6-Assumptions!B62)</f>
+        <v/>
+      </c>
+      <c r="C140" s="9">
+        <f>550*(Assumptions!B6-Assumptions!B62)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v5.0: survey card cleaned up with sampling statistics; one late family added
The survey results card is restructured for readability: the cleaned
counts up front (38 households / 85 children after duplicate removal,
including one family with one child received after the form closed),
the results table, what the answers add up to, and a dedicated
sampling-statistics note (24 of ~115-128 enrolled sampled, 20-of-24
raw split, the response-propensity correction and its posterior).

The added family moves the floor from 73 to 74 students ($377,354 a
year) and the grid re-bases: median -$293,756, middle half -$489,057
to -$113,244, default -$315,285. Every artifact, chart, and test pin
re-based; the statistical band is unchanged (the child is not yet
enrolled, so the enrolled-sample split stays 20 of 24).

Suites: validate 734/0, sync 73/0, site 0 failures.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -1156,7 +1156,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$292,348 at Closure_Model row 50)</t>
+          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$293,756 at Closure_Model row 50)</t>
         </is>
       </c>
       <c r="B21" s="26">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F46" s="21" t="inlineStr">
         <is>
-          <t>Above the closure model's central case, which is itself negative (-$299,327); the weighted median loses $292,348</t>
+          <t>Above the closure model's central case, which is itself negative (-$299,327); the weighted median loses $293,756</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>-292348</v>
+        <v>-293756</v>
       </c>
       <c r="C47" s="9">
         <f>B47*(1-(1+B$40)^-B$41)/B$40</f>
@@ -2844,7 +2844,7 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Closure range check (v5.0): at the +$409,190 best case FY2029 holds a modest cushion; at the -$292,348 weighted median the reserves go MUCH faster than status quo; 88 percent of weighted scenarios lose money and drain reserves faster than doing nothing.</t>
+          <t>Closure range check (v5.0): at the +$409,190 best case FY2029 holds a modest cushion; at the -$293,756 weighted median the reserves go MUCH faster than status quo; 88 percent of weighted scenarios lose money and drain reserves faster than doing nothing.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-292348</v>
+        <v>-293756</v>
       </c>
       <c r="C6" s="9">
         <f>Runway!E7</f>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Closure vote; the weighted median LOSES $292,348 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $299,327, and even the +$409,190 best-case tail covers only 15.4% of the $2.65M gap; longer rides; measured enrollment-loss risk</t>
+          <t>Closure vote; the weighted median LOSES $293,756 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $299,327, and even the +$409,190 best-case tail covers only 15.4% of the $2.65M gap; longer rides; measured enrollment-loss risk</t>
         </is>
       </c>
     </row>
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="B35" s="9">
-        <f>-292348/Assumptions!B11</f>
+        <f>-293756/Assumptions!B11</f>
         <v/>
       </c>
       <c r="C35" s="9">
@@ -11190,11 +11190,11 @@
         </is>
       </c>
       <c r="B34" s="19">
-        <f>B17+C17-63000-73*(Assumptions!B6+500)</f>
+        <f>B17+C17-63000-74*(Assumptions!B6+500)</f>
         <v/>
       </c>
       <c r="F34" s="21">
-        <f> $127,039 kept, minus $63,000 of busing, minus the survey floor of 73 missing students at $5,126 with nothing shed: the published -$310,159, the 47th percentile of the 14,580-scenario grid; the weighted median is a $292,348 loss (Closure_Model row 50)</f>
+        <f> $127,039 kept, minus $63,000 of busing, minus the survey floor of 74 missing students at $5,126 with nothing shed: the published -$315,285, the 47th percentile of the 14,580-scenario grid; the weighted median is a $293,756 loss (Closure_Model row 50)</f>
         <v/>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 14,580-scenario grid at row 37, median a $292,348 LOSS)</t>
+          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 14,580-scenario grid at row 37, median a $293,756 LOSS)</t>
         </is>
       </c>
       <c r="B20" s="28">
@@ -12575,7 +12575,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Students missing from the rolls at steady state (grid legs 38/73/137/167/194)</t>
+          <t>Students missing from the rolls at steady state (grid legs 38/74/137/167/194)</t>
         </is>
       </c>
       <c r="B43" s="10" t="n">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>From the August 2026 school-choice survey (anonymized in build/) and build/exodus_model.py: 73 = the floor, 30 signed households' 69 children at 5.75 per class x 12.62 effective years of the district's own grade-to-grade survival; 137/167/194 = the response-bias-corrected posterior quartiles at the class midpoint; 38 = half the floor, the skeptic's leg. Exits free and funded under HB 563. The state's SAAR files corroborate: kindergarten 12 in 2025-26 against a 21-31 norm; end-of-year 141/128/115 across 2023-24 to 2025-26.</t>
+          <t>From the August 2026 school-choice survey (anonymized in build/) and build/exodus_model.py: 74 = the floor, 31 signed households' 70 children at 5.83 per class x 12.62 effective years of the district's own grade-to-grade survival; 137/167/194 = the response-bias-corrected posterior quartiles at the class midpoint; 38 = roughly half the floor, the skeptic's leg. Exits free and funded under HB 563. The state's SAAR files corroborate: kindergarten 12 in 2025-26 against a 21-31 norm; end-of-year 141/128/115 across 2023-24 to 2025-26.</t>
         </is>
       </c>
     </row>
@@ -12707,7 +12707,7 @@
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>Distribution of all 14,580 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, shed, property and busing levers take three values each, teachers four (0/1/2/3) and missing students five (38/73/137/167/194): 3^6 x 4 x 5 = 14,580. v5.0 lever weights: triangular 1-2-1 on the six levers with a documented central setting; uniform on teachers; survey-anchored 1-2-2-2-1 on missing students. Weighted median -$292,348 (the median scenario LOSES money); middle half -$488,920 to -$111,080; 88 percent of weighted scenarios negative; range -$1,322,925 to +$409,190 (unweighted median -$283,934). REBUILT IN v5.0 on the August 2026 school-choice survey: the leaver lever moves from guessed shares of 128 (0-64, year one only) to measured students missing at steady state, and the new shed lever nets the district's cost response against each lost student's SEEK. One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
+          <t>Distribution of all 14,580 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, shed, property and busing levers take three values each, teachers four (0/1/2/3) and missing students five (38/74/137/167/194): 3^6 x 4 x 5 = 14,580. v5.0 lever weights: triangular 1-2-1 on the six levers with a documented central setting; uniform on teachers; survey-anchored 1-2-2-2-1 on missing students. Weighted median -$293,756 (the median scenario LOSES money); middle half -$489,057 to -$113,244; 88 percent of weighted scenarios negative; range -$1,322,925 to +$409,190 (unweighted median -$284,962). REBUILT IN v5.0 on the August 2026 school-choice survey: the leaver lever moves from guessed shares of 128 (0-64, year one only) to measured students missing at steady state, and the new shed lever nets the district's cost response against each lost student's SEEK. One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
         </is>
       </c>
     </row>
@@ -12845,10 +12845,10 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C5" s="10" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6">
@@ -12858,10 +12858,10 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>5.75 out of every class of 19 to 24 (recent SAAR grade range)</t>
+          <t>5.83 out of every class of 19 to 24 (recent SAAR grade range)</t>
         </is>
       </c>
     </row>
@@ -13032,7 +13032,7 @@
       </c>
       <c r="F19" s="21" t="inlineStr">
         <is>
-          <t>The 30 signed households alone: no statistics. $371,963 a year.</t>
+          <t>The 31 signed households alone: no statistics. $377,354 a year.</t>
         </is>
       </c>
     </row>
@@ -14509,7 +14509,7 @@
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $1,322,925 to plus $409,190 with a weighted median of minus $292,348, and not the school's $2.5M gross cost.</t>
+          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $1,322,925 to plus $409,190 with a weighted median of minus $293,756, and not the school's $2.5M gross cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.0: closure calculator opens at the statistical median of leavers
The default scenario keeps the district's all-staff-retained stance but
prices families leaving at the selection-corrected median (167 students
a year) instead of the survey floor (74). Default net moves from a
$286,425 loss to a $726,873 loss, the 16th percentile of the 4,860
weighted scenarios; the tax-equivalent line moves to about 4.4 cents.
Site, grid script, model Defaults tab, report version history, and all
three test suites updated together.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -11186,15 +11186,15 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Closure default: district staffing stance + the survey floor of missing students</t>
+          <t>Closure default: district staffing stance + the statistical median of missing students</t>
         </is>
       </c>
       <c r="B34" s="19">
-        <f>B17+C17-63000-74*(Assumptions!B6+500-Assumptions!B62)</f>
+        <f>B17+C17-63000-167*(Assumptions!B6+500-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="F34" s="21">
-        <f> $127,039 kept, minus $63,000 of busing, minus the survey floor of 74 missing students at $5,136 less the $400 supplies credit: the published -$286,425, the 68th percentile of the 4,860-scenario grid; the weighted median is a $474,042 loss (Closure_Model row 50)</f>
+        <f> $127,039 kept, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$726,873, the 16th percentile of the 4,860-scenario grid; the weighted median is a $474,042 loss (Closure_Model row 50)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.0: calculator opens at the savings-granted case
The default closure scenario now grants every saving that scales with
students: the $400 supplies credit per missing child (already in the
leaver term), three teachers cut with the emptied classrooms (the most
the district's own classroom count supports), and half of the fixed
overhead positions cut over time, priced against the statistical median
of 167 students leaving. Default net moves from a $726,873 loss (all
staff retained) to a $456,383 loss at the 59th percentile of the 3,888
weighted scenarios; the tax-equivalent line moves to about 2.7 cents.
The grid script's printed rank now half-weights ties, matching the site
JS convention. Site, grid script, model Defaults tab, report version
history, and all three test suites updated together.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -11186,15 +11186,15 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Closure default: district staffing stance + the statistical median of missing students</t>
+          <t>Closure default: scaled savings granted (teachers included, half the fixed overhead) + the statistical median of missing students</t>
         </is>
       </c>
       <c r="B34" s="19">
-        <f>B17+C17-63000-167*(Assumptions!B6+500-Assumptions!B62)</f>
+        <f>B17+C17+Closure_Model!C40+3*54479.4-63000-167*(Assumptions!B6+500-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="F34" s="21">
-        <f> $127,039 kept, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$726,873, the 19th percentile of the 3,888-scenario grid; the weighted median is a $523,830 loss (Closure_Model row 50)</f>
+        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$456,383, the 59th percentile of the 3,888-scenario grid; the weighted median is a $523,830 loss (Closure_Model row 50)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.0: six-lever grid; busing high leg halved, property lever removed
The busing lever's high leg is capped at half its bottom-up maximum
($190,000 to $95,000) and the speculative property-value lever is
removed while the PVA records request is pending; the community research
on property effects stays in the report's Section 6 but is no longer
priced. The grid tightens from 3,888 to 1,296 scenarios and every
statistic moves in closure's favor while the conclusion holds: weighted
median loss $456,383 a year, middle half $606,202 to $241,706, 97
percent of scenarios lose money, range -$1,057,265 to +$171,118, central
case -$415,542. The savings-granted calculator default (-$456,383) is
now exactly the grid's weighted median scenario, at the 50th percentile.
Site, grid script, charts, PDF, summary, workbook, and all three test
suites updated together.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -1156,7 +1156,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$523,830 at Closure_Model row 50)</t>
+          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$456,383 at Closure_Model row 50)</t>
         </is>
       </c>
       <c r="B21" s="26">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F46" s="21" t="inlineStr">
         <is>
-          <t>Above the closure model's central case, which is itself negative (-$463,042); the weighted median loses $523,830</t>
+          <t>Above the closure model's central case, which is itself negative (-$415,542); the weighted median loses $456,383</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>-523830</v>
+        <v>-456383</v>
       </c>
       <c r="C47" s="9">
         <f>B47*(1-(1+B$40)^-B$41)/B$40</f>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="F47" s="21" t="inlineStr">
         <is>
-          <t>Closure_Model tab, 3,888-combination grid; the median scenario loses money</t>
+          <t>Closure_Model tab, 1,296-combination grid; the median scenario loses money</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Closure range check (v5.0): at the +$171,118 best case FY2029 holds a modest cushion; at the -$523,830 weighted median the reserves go MUCH faster than status quo; 99 percent of weighted scenarios lose money and drain reserves faster than doing nothing.</t>
+          <t>Closure range check (v5.0): at the +$171,118 best case FY2029 holds a modest cushion; at the -$456,383 weighted median the reserves go MUCH faster than status quo; 97 percent of weighted scenarios lose money and drain reserves faster than doing nothing.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-523830</v>
+        <v>-456383</v>
       </c>
       <c r="C6" s="9">
         <f>Runway!E7</f>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Closure vote; the weighted median LOSES $523,830 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $463,042, and even the +$171,118 best-case tail covers only 6.5% of the $2.65M gap; longer rides; measured enrollment-loss risk</t>
+          <t>Closure vote; the weighted median LOSES $456,383 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $415,542, and even the +$171,118 best-case tail covers only 6.5% of the $2.65M gap; longer rides; measured enrollment-loss risk</t>
         </is>
       </c>
     </row>
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="B35" s="9">
-        <f>-523830/Assumptions!B11</f>
+        <f>-456383/Assumptions!B11</f>
         <v/>
       </c>
       <c r="C35" s="9">
@@ -11194,7 +11194,7 @@
         <v/>
       </c>
       <c r="F34" s="21">
-        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$456,383, the 59th percentile of the 3,888-scenario grid; the weighted median is a $523,830 loss (Closure_Model row 50)</f>
+        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$456,383, which is also the weighted median of the 1,296-scenario grid (Closure_Model row 50)</f>
         <v/>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 3,888-scenario grid at row 37, median a $523,830 LOSS)</t>
+          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 1,296-scenario grid at row 37, median a $456,383 LOSS)</t>
         </is>
       </c>
       <c r="B20" s="28">
@@ -12457,7 +12457,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>V5.0 TWO-TAILED SENSITIVITY: SEVEN LEVERS, 3,888 COMBINATIONS (backs Figure 5; THIS GRID, not the legacy single-point rows above, is the published closure model)</t>
+          <t>V5.0 TWO-TAILED SENSITIVITY: SIX LEVERS, 1,296 COMBINATIONS (backs Figure 5; THIS GRID, not the legacy single-point rows above, is the published closure model)</t>
         </is>
       </c>
     </row>
@@ -12564,11 +12564,11 @@
         <v>63000</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>190000</v>
+        <v>95000</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Derived bottom-up with uncertainty: 2-4 zone buses terminating in Paris (~9-11 road miles farther one-way), 2 loaded + 0-2 deadhead legs daily, 170 to 175 days, $3.25-$4.75/mile (KDE/NAPT band), high stop adds one $45,000 route split. Per zone student $160/$492/$1,495 vs the $1,032 district average. The July 2026 records response produced the current routes but answered N/A for any routing study or ride-time analysis.</t>
+          <t>Derived bottom-up with uncertainty: 2-4 zone buses terminating in Paris (~9-11 road miles farther one-way), 2 loaded + 0-2 deadhead legs daily, 170 to 175 days, $3.25-$4.75/mile (KDE/NAPT band). The bottom-up maximum with a route split reached $190,000; v5.0 caps the high leg at half that, $95,000. The July 2026 records response produced the current routes but answered N/A for any routing study or ride-time analysis.</t>
         </is>
       </c>
     </row>
@@ -12614,27 +12614,6 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>Property-value loss (zone tax base)</t>
-        </is>
-      </c>
-      <c r="B45" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" s="8" t="n">
-        <v>47500</v>
-      </c>
-      <c r="D45" s="8" t="n">
-        <v>95000</v>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Roughly 0-10 percent of an estimated zone base; kept as foregone revenue because the board's rate practice does not raise rates to recapture zone valuation losses; PVA records ask pending</t>
-        </is>
-      </c>
-    </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -12642,12 +12621,12 @@
         </is>
       </c>
       <c r="B47" s="19">
-        <f>C39+C40+C41*54479.4-C42-C43*(Assumptions!B6+C44-Assumptions!B62)-C45</f>
+        <f>C39+C40+C41*54479.4-C42-C43*(Assumptions!B6+C44-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>-$463,042: the central case itself loses money, about 17 percent of the structural deficit added, not removed</t>
+          <t>-$415,542: the central case itself loses money, about 16 percent of the structural deficit added, not removed</t>
         </is>
       </c>
     </row>
@@ -12658,12 +12637,12 @@
         </is>
       </c>
       <c r="B48" s="9">
-        <f>B39+B40+B41*54479.4-D42-D43*(Assumptions!B6+D44-Assumptions!B62)-D45</f>
+        <f>B39+B40+B41*54479.4-D42-D43*(Assumptions!B6+D44-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>-$1,247,265 a year: the closure loses money</t>
+          <t>-$1,057,265 a year: the closure loses money</t>
         </is>
       </c>
     </row>
@@ -12674,7 +12653,7 @@
         </is>
       </c>
       <c r="B49" s="9">
-        <f>D39+D40+D41*54479.4-B42-B43*(Assumptions!B6+B44-Assumptions!B62)-B45</f>
+        <f>D39+D40+D41*54479.4-B42-B43*(Assumptions!B6+B44-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -12686,7 +12665,7 @@
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>Distribution of all 3,888 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, property and busing levers take three values each, teachers four (0/1/2/3) and missing students four (74/137/167/194): 3^5 x 4 x 4 = 3,888. Each missing student is priced at the enacted FY2027 SEEK base of $4,636 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. v5.0 lever weights: triangular 1-2-1 on the five levers with a documented central setting; uniform on teachers; survey-anchored 2-2-2-1 on missing students, the signed-survey floor held as the low end. Weighted median -$523,830 (the median scenario LOSES money); middle half -$681,643 to -$314,250; 99 percent of weighted scenarios negative; range -$1,247,265 to +$171,118 (unweighted median -$562,162). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
+          <t>Distribution of all 1,296 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons and busing levers take three values each, teachers four (0/1/2/3) and missing students four (74/137/167/194): 3^4 x 4 x 4 = 1,296. Each missing student is priced at the enacted FY2027 SEEK base of $4,636 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending. v5.0 lever weights: triangular 1-2-1 on the four levers with a documented central setting; uniform on teachers; survey-anchored 2-2-2-1 on missing students, the signed-survey floor held as the low end. Weighted median -$456,383 (the median scenario LOSES money, and the website default IS this median scenario); middle half -$606,202 to -$241,706; 97 percent of weighted scenarios negative; range -$1,057,265 to +$171,118 (unweighted median -$488,532). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
         </is>
       </c>
     </row>
@@ -13147,7 +13126,7 @@
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>Teacher savings are priced ONLY on the Closure_Model teachers-cut lever (the district's own 0 to 3 positions), never here, so staffing savings cannot be counted twice. Even with the supplies credit and the teacher lever at its friendliest, 99 percent of priced closure scenarios lose money.</t>
+          <t>Teacher savings are priced ONLY on the Closure_Model teachers-cut lever (the district's own 0 to 3 positions), never here, so staffing savings cannot be counted twice. Even with the supplies credit and the teacher lever at its friendliest, 97 percent of priced closure scenarios lose money.</t>
         </is>
       </c>
     </row>
@@ -14455,7 +14434,7 @@
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $1,247,265 to plus $171,118 with a weighted median of minus $523,830, and not the school's $2.5M gross cost.</t>
+          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $1,057,265 to plus $171,118 with a weighted median of minus $456,383, and not the school's $2.5M gross cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v5.0: leaver lever prices the statistical band's middle half
The survey-floor leg (74) leaves the grid: the students-missing lever is
now triangular on the selection-corrected posterior quartiles alone
(137/167/194), matching every other centered lever, and the signed floor
stays in Section 5 as hard evidence rather than a priced scenario. The
grid tightens from 1,296 to 972 scenarios and the conclusion sharpens:
EVERY priced scenario loses money. Weighted median loss $571,883 a year,
middle half $679,361 to $467,862, range -$1,057,265 to -$95,750 (the
best case, all six levers closure-friendly, still loses $95,750),
central case -$557,622. The savings-granted default (-$456,383) sits at
the 77th percentile, friendlier than three quarters of the grid. Site,
grid script, charts, PDF, summary, workbook, and all three test suites
updated together.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -1156,7 +1156,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$456,383 at Closure_Model row 50)</t>
+          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$571,883 at Closure_Model row 50)</t>
         </is>
       </c>
       <c r="B21" s="26">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F46" s="21" t="inlineStr">
         <is>
-          <t>Above the closure model's central case, which is itself negative (-$415,542); the weighted median loses $456,383</t>
+          <t>Above the closure model's central case, which is itself negative (-$557,622); the weighted median loses $571,883</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>-456383</v>
+        <v>-571883</v>
       </c>
       <c r="C47" s="9">
         <f>B47*(1-(1+B$40)^-B$41)/B$40</f>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="F47" s="21" t="inlineStr">
         <is>
-          <t>Closure_Model tab, 1,296-combination grid; the median scenario loses money</t>
+          <t>Closure_Model tab, 972-combination grid; the median scenario loses money</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Closure range check (v5.0): at the +$171,118 best case FY2029 holds a modest cushion; at the -$456,383 weighted median the reserves go MUCH faster than status quo; 97 percent of weighted scenarios lose money and drain reserves faster than doing nothing.</t>
+          <t>Closure range check (v5.0): even the -$95,750 best case drains reserves faster than status quo, the -$571,883 weighted median much faster; every weighted scenario loses money.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-456383</v>
+        <v>-571883</v>
       </c>
       <c r="C6" s="9">
         <f>Runway!E7</f>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Closure vote; the weighted median LOSES $456,383 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $415,542, and even the +$171,118 best-case tail covers only 6.5% of the $2.65M gap; longer rides; measured enrollment-loss risk</t>
+          <t>Closure vote; the weighted median LOSES $571,883 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $557,622, and even the best-case tail still loses $95,750 a year; longer rides; measured enrollment-loss risk</t>
         </is>
       </c>
     </row>
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="B35" s="9">
-        <f>-456383/Assumptions!B11</f>
+        <f>-571883/Assumptions!B11</f>
         <v/>
       </c>
       <c r="C35" s="9">
@@ -11194,7 +11194,7 @@
         <v/>
       </c>
       <c r="F34" s="21">
-        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$456,383, which is also the weighted median of the 1,296-scenario grid (Closure_Model row 50)</f>
+        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 167 missing students at $5,136 less the $400 supplies credit: the published -$456,383, the 77th percentile of the 972-scenario grid; the weighted median is a $571,883 loss (Closure_Model row 50)</f>
         <v/>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 1,296-scenario grid at row 37, median a $456,383 LOSS)</t>
+          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 972-scenario grid at row 37, median a $571,883 LOSS)</t>
         </is>
       </c>
       <c r="B20" s="28">
@@ -12457,7 +12457,7 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>V5.0 TWO-TAILED SENSITIVITY: SIX LEVERS, 1,296 COMBINATIONS (backs Figure 5; THIS GRID, not the legacy single-point rows above, is the published closure model)</t>
+          <t>V5.0 TWO-TAILED SENSITIVITY: SIX LEVERS, 972 COMBINATIONS (backs Figure 5; THIS GRID, not the legacy single-point rows above, is the published closure model)</t>
         </is>
       </c>
     </row>
@@ -12575,21 +12575,21 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Students missing from the rolls at steady state (grid legs 74/137/167/194)</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="n">
-        <v>74</v>
+          <t>Students missing from the rolls at steady state (grid legs 137/167/194)</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="n">
+        <v>137</v>
       </c>
       <c r="C43" s="8" t="n">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="D43" s="8" t="n">
         <v>194</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>From the August 2026 school-choice survey (anonymized in build/) and build/exodus_model.py: 74 = the floor, 31 signed households' 70 children at 5.83 per class x 12.62 effective years of the district's own grade-to-grade survival; 137/167/194 = the response-bias-corrected posterior quartiles at the class midpoint. The floor is the grid's low end: fewer leavers than the signed households account for is not a priced scenario. Exits free and funded under HB 563. The state's SAAR files corroborate: kindergarten 12 in 2025-26 against a 21-31 norm; end-of-year 141/128/115 across 2023-24 to 2025-26.</t>
+          <t>From the August 2026 school-choice survey (anonymized in build/) and build/exodus_model.py: 74 = the floor, 31 signed households' 70 children at 5.83 per class x 12.62 effective years of the district's own grade-to-grade survival; 137/167/194 = the response-bias-corrected posterior 25th/50th/75th percentiles at the class midpoint, triangular with the median central. The signed-survey floor of 74 (31 households, 70 children, 5.83 per class x 12.62 effective years) sits below every priced leg and is kept as hard evidence, not as a scenario. Exits free and funded under HB 563. The state's SAAR files corroborate: kindergarten 12 in 2025-26 against a 21-31 norm; end-of-year 141/128/115 across 2023-24 to 2025-26.</t>
         </is>
       </c>
     </row>
@@ -12626,7 +12626,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>-$415,542: the central case itself loses money, about 16 percent of the structural deficit added, not removed</t>
+          <t>-$557,622: the central case itself loses money, about 21 percent of the structural deficit added, not removed</t>
         </is>
       </c>
     </row>
@@ -12658,14 +12658,14 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>+$171,118 a year: the grid's best case (every lever at its closure-friendliest, only the survey-floor leavers the signed households account for), still below the plan's $800K-$1M requirement</t>
+          <t>-$95,750 a year: even the grid's best case (every lever at its closure-friendliest, the band's low leg of 137 leavers) loses money, roughly $900,000 to $1.1 million short of the plan's $800K-$1M requirement</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>Distribution of all 1,296 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons and busing levers take three values each, teachers four (0/1/2/3) and missing students four (74/137/167/194): 3^4 x 4 x 4 = 1,296. Each missing student is priced at the enacted FY2027 SEEK base of $4,636 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending. v5.0 lever weights: triangular 1-2-1 on the four levers with a documented central setting; uniform on teachers; survey-anchored 2-2-2-1 on missing students, the signed-survey floor held as the low end. Weighted median -$456,383 (the median scenario LOSES money, and the website default IS this median scenario); middle half -$606,202 to -$241,706; 97 percent of weighted scenarios negative; range -$1,057,265 to +$171,118 (unweighted median -$488,532). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
+          <t>Distribution of all 972 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, busing and missing-students levers take three values each, teachers four (0/1/2/3): 3^5 x 4 = 972. Each missing student is priced at the enacted FY2027 SEEK base of $4,636 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending; the missing-students lever prices the statistical band's quartiles (137/167/194), with the signed-survey floor of 74 kept as hard evidence below every priced leg. v5.0 lever weights: triangular 1-2-1 on every three-leg lever, uniform on teachers. Weighted median -$571,883 (the median scenario LOSES money); middle half -$679,361 to -$467,862; EVERY weighted scenario is negative, the best case still loses $95,750; range -$1,057,265 to -$95,750 (unweighted median -$566,628). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
         </is>
       </c>
     </row>
@@ -13126,7 +13126,7 @@
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>Teacher savings are priced ONLY on the Closure_Model teachers-cut lever (the district's own 0 to 3 positions), never here, so staffing savings cannot be counted twice. Even with the supplies credit and the teacher lever at its friendliest, 97 percent of priced closure scenarios lose money.</t>
+          <t>Teacher savings are priced ONLY on the Closure_Model teachers-cut lever (the district's own 0 to 3 positions), never here, so staffing savings cannot be counted twice. Even with the supplies credit and the teacher lever at its friendliest, every priced closure scenario loses money.</t>
         </is>
       </c>
     </row>
@@ -14434,7 +14434,7 @@
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $1,057,265 to plus $171,118 with a weighted median of minus $456,383, and not the school's $2.5M gross cost.</t>
+          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $1,057,265 to minus $95,750 with a weighted median of minus $571,883, and not the school's $2.5M gross cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Widen the survey evidence window: current enrollment plus the next three entering classes
Per review of the hand-coded class years: the sample now spans K-2020
through K-2028, so a miscoded child counts either way. 62 of 75 would
leave (83 percent), corrected by the same truncated response-bias prior
(k >= 3.3). New posterior band 43 to 57 percent, median 50; steady-state
legs 117/136/154 students ($600,912/$698,496/$790,944). The closure grid
tightens and every one of the 972 scenarios loses money again: weighted
median -$428,627, middle half -$519,765 to -$340,021, range -$847,825
to -$11,030, site default -$309,567 at the 82nd percentile. Site,
summary, workbook, charts, and tests all rebased; browser suite green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -1156,7 +1156,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$447,573 at Closure_Model row 50)</t>
+          <t>Closure net saving (LEGACY single-point base case, superseded by the grid median of -$428,627 at Closure_Model row 50)</t>
         </is>
       </c>
       <c r="B21" s="26">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="F46" s="21" t="inlineStr">
         <is>
-          <t>Above the closure model's central case, which is itself negative (-$429,750); the weighted median loses $447,573</t>
+          <t>Above the closure model's central case, which is itself negative (-$410,806); the weighted median loses $428,627</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>-447573</v>
+        <v>-428627</v>
       </c>
       <c r="C47" s="9">
         <f>B47*(1-(1+B$40)^-B$41)/B$40</f>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>1678</v>
+        <v>-11030</v>
       </c>
       <c r="C48" s="9">
         <f>B48*(1-(1+B$40)^-B$41)/B$40</f>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="F48" s="21" t="inlineStr">
         <is>
-          <t>Closure_Model tab B49: the grid's lone positive corner</t>
+          <t>Closure_Model tab B49</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Closure range check (v5.0): the grid's lone positive corner (+$1,678) is a rounding error against the need; the -$447,573 weighted median drains reserves faster than status quo; all but one of the 972 weighted scenarios lose money.</t>
+          <t>Closure range check (v5.0): even the -$11,030 best case drains reserves faster than status quo, the -$428,627 weighted median much faster; every weighted scenario loses money.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>-447573</v>
+        <v>-428627</v>
       </c>
       <c r="C6" s="9">
         <f>Runway!E7</f>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Closure vote; the weighted median LOSES $447,573 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $429,750, and 971 of the 972 weighted scenarios lose money (the lone best corner nets $1,678); longer rides; measured enrollment-loss risk</t>
+          <t>Closure vote; the weighted median LOSES $428,627 a year (B6 is the grid median; the legacy single-point Closure_Model!B20 is superseded); the grid central case itself loses $410,806, and even the best-case tail still loses $11,030 a year; longer rides; measured enrollment-loss risk</t>
         </is>
       </c>
     </row>
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="B35" s="9">
-        <f>-447573/Assumptions!B11</f>
+        <f>-428627/Assumptions!B11</f>
         <v/>
       </c>
       <c r="C35" s="9">
@@ -11190,11 +11190,11 @@
         </is>
       </c>
       <c r="B34" s="19">
-        <f>B17+C17+Closure_Model!C40+3*54479.4-63000-140*(Assumptions!B6+500-Assumptions!B62)</f>
+        <f>B17+C17+Closure_Model!C40+3*54479.4-63000-136*(Assumptions!B6+500-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="F34" s="21">
-        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 140 missing students at $5,136 less the $400 supplies credit: the published -$328,511, the 79th percentile of the 972-scenario grid; the weighted median is a $447,573 loss (Closure_Model row 50)</f>
+        <f> $127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 136 missing students at $5,136 less the $400 supplies credit: the published -$309,567, the 82nd percentile of the 972-scenario grid; the weighted median is a $428,627 loss (Closure_Model row 50)</f>
         <v/>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 972-scenario grid at row 37, median a $447,573 LOSS)</t>
+          <t>NET RECURRING GENERAL FUND SAVING (LEGACY single-point scenario on superseded inputs; the published model is the 972-scenario grid at row 37, median a $428,627 LOSS)</t>
         </is>
       </c>
       <c r="B20" s="28">
@@ -12575,17 +12575,17 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Students missing from the rolls at steady state (grid legs 114/140/167)</t>
+          <t>Students missing from the rolls at steady state (grid legs 117/136/154)</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C43" s="8" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>167</v>
+        <v>154</v>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
@@ -12626,7 +12626,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>-$429,750: the central case itself loses money, about 16 percent of the structural deficit added, not removed</t>
+          <t>-$410,806: the central case itself loses money, about 16 percent of the structural deficit added, not removed</t>
         </is>
       </c>
     </row>
@@ -12642,7 +12642,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>-$915,893 a year: the closure loses money</t>
+          <t>-$847,825 a year: the closure loses money</t>
         </is>
       </c>
     </row>
@@ -12658,14 +12658,14 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>+$1,678 a year: the grid's single positive cell (every lever at its closure-friendliest at once: full capture, every fixed position cut, three teachers, only 114 leavers with zero add-ons, minimal busing), about $13 per displaced student and $800,000 to $1 million short of the plan's requirement</t>
+          <t>-$11,030 a year: even the grid's best case (every lever at its closure-friendliest at once) still loses money, roughly $800,000 to $1 million short of the plan's requirement</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>Distribution of all 972 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, busing and missing-students levers take three values each, teachers four (0/1/2/3): 3^5 x 4 = 972. Each missing student is priced at the enacted FY2027 SEEK base of $4,636 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending; the missing-students lever prices the statistical band's quartiles (114/140/167), with the signed-survey floor of 74 kept as hard evidence below every priced leg. v5.0 lever weights: triangular 1-2-1 on every three-leg lever, uniform on teachers. Weighted median -$447,573 (the median scenario LOSES money); middle half -$552,323 to -$347,374; all but ONE of the 972 weighted scenarios are negative, and the single best corner nets +$1,678 a year, about $13 per displaced student; range -$915,893 to +$1,678 (unweighted median -$446,722). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
+          <t>Distribution of all 972 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, busing and missing-students levers take three values each, teachers four (0/1/2/3): 3^5 x 4 = 972. Each missing student is priced at the enacted FY2027 SEEK base of $4,636 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending; the missing-students lever prices the statistical band's quartiles (117/136/154), with the signed-survey floor of 74 kept as hard evidence below every priced leg. v5.0 lever weights: triangular 1-2-1 on every three-leg lever, uniform on teachers. Weighted median -$428,627 (the median scenario LOSES money); middle half -$519,765 to -$340,021; EVERY weighted scenario is negative, the best case still loses $11,030; range -$847,825 to -$11,030 (unweighted median -$426,503). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
         </is>
       </c>
     </row>
@@ -12971,7 +12971,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>0.42025</v>
+        <v>0.42975</v>
       </c>
       <c r="C19" s="11">
         <f>ROUND(B19*$B$8,0)</f>
@@ -12998,7 +12998,7 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>0.51625</v>
+        <v>0.50075</v>
       </c>
       <c r="C20" s="11">
         <f>ROUND(B20*$B$8,0)</f>
@@ -13025,7 +13025,7 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>0.61375</v>
+        <v>0.56725</v>
       </c>
       <c r="C21" s="11">
         <f>ROUND(B21*$B$8,0)</f>
@@ -13052,7 +13052,7 @@
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>0.74475</v>
+        <v>0.65525</v>
       </c>
       <c r="C22" s="11">
         <f>ROUND(B22*$B$8,0)</f>
@@ -13075,7 +13075,7 @@
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>Leave shares are the posterior of a response-propensity model: among enrolled surveyed children the raw split is 20 leavers to 4 stayers; leaving families are assumed 3.3x to about 9x likelier to answer (log-normal prior centered on 3.5x and FLOORED at 3.3x, the lower of Pew's high-salience benchmarks, chosen for a small, emotionally charged respondent pool reached through a campaign-circulated form), and the shares above are the resulting quartiles. The 24-child enrolled sample is the hand-coded floor: class-year designations are not assumed accurate and likely undercount who is enrolled now, so the true enrolled respondent count is probably higher at a similar leave rate, and the silent pool smaller than the correction assumes; both effects would raise the corrected share, so the published band leans low. Corroboration outside the survey: SAAR 2025-26 kindergarten of 12 against a ten-year average of 22; end-of-year 141 / 128 / 115 across 2023-24 to 2025-26. Losses build from six grade cohorts in year one to all thirteen by year eight (141 of 169 cohort-years across a 13-year window).</t>
+          <t>Leave shares are the posterior of a response-propensity model: across the sampled window the raw split is 62 leavers to 13 stayers; leaving families are assumed 3.3x to about 9x likelier to answer (log-normal prior centered on 3.5x and FLOORED at 3.3x, the lower of Pew's high-salience benchmarks, chosen for a small, emotionally charged respondent pool reached through a campaign-circulated form), and the shares above are the resulting quartiles. Class-year codes are not assumed accurate; the evidence window spans current enrollment plus the next three entering classes (62 leavers to 13 stayers of 75), so a miscoded child counts either way, and the correction still assumes the largest silent pool the coding allows, leaning the band low. Corroboration outside the survey: SAAR 2025-26 kindergarten of 12 against a ten-year average of 22; end-of-year 141 / 128 / 115 across 2023-24 to 2025-26. Losses build from six grade cohorts in year one to all thirteen by year eight (141 of 169 cohort-years across a 13-year window).</t>
         </is>
       </c>
     </row>
@@ -14408,7 +14408,7 @@
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $915,893 to plus $1,678 with a weighted median of minus $447,573, and not the school's $2.5M gross cost.</t>
+          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $847,825 to minus $11,030 with a weighted median of minus $428,627, and not the school's $2.5M gross cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restate the today baseline on the 2025-26 end-of-year count of 115
The exodus ladder, survey share-of-school tables, and per-displaced
figures now use 115, the newest official SAAR end-of-year count: today's
band 49 to 65 students ($251,664 to $333,840 a year, median 58), the 70
signed-out children equal 61 percent of enrollment, the closure median is
$3,727 per displaced student and the plan requirement $6,957 to $8,696.
Capacity and cost comparisons keep the official 2024-25 filings at 128,
relabeled where they said today. Steady state and the 972-scenario grid
are unchanged. Disclosed in the version history. All suites green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -8768,15 +8768,15 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Plan requirement, low / high ($800K-$1M over the 128 students displaced)</t>
+          <t>Plan requirement, low / high ($800K-$1M over the 115 students displaced, the 2025-26 end-of-year count)</t>
         </is>
       </c>
       <c r="B34" s="19">
-        <f>800000/Assumptions!B11</f>
+        <f>800000/Exodus_Model!B8</f>
         <v/>
       </c>
       <c r="C34" s="19">
-        <f>1000000/Assumptions!B11</f>
+        <f>1000000/Exodus_Model!B8</f>
         <v/>
       </c>
     </row>
@@ -8787,15 +8787,15 @@
         </is>
       </c>
       <c r="B35" s="9">
-        <f>-428627/Assumptions!B11</f>
+        <f>-428627/Exodus_Model!B8</f>
         <v/>
       </c>
       <c r="C35" s="9">
-        <f>Closure_Model!B47/Assumptions!B11</f>
+        <f>Closure_Model!B47/Exodus_Model!B8</f>
         <v/>
       </c>
       <c r="D35" s="9">
-        <f>Closure_Model!B49/Assumptions!B11</f>
+        <f>Closure_Model!B49/Exodus_Model!B8</f>
         <v/>
       </c>
     </row>
@@ -8881,14 +8881,14 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>BRACKET CHECK (v3.9): the record's plausible median vs this model's independent bottom-up median per displaced student. These bracket rather than coincide and measure different things: the record credits a district's whole budget change to its closure (an upper bound by construction), the model prices only the levers a closure moves. Before the v3.9 fixed-cost rebuild the model read $713 and the two nearly coincided. Both remain far below the plan's $6,250-$7,813 requirement.</t>
+          <t>BRACKET CHECK (v3.9): the record's plausible median vs this model's independent bottom-up median per displaced student. These bracket rather than coincide and measure different things: the record credits a district's whole budget change to its closure (an upper bound by construction), the model prices only the levers a closure moves. Before the v3.9 fixed-cost rebuild the model read $713 and the two nearly coincided. Both remain far below the plan's $6,957-$8,696 requirement.</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
         <v>818</v>
       </c>
       <c r="C44" s="19">
-        <f>Closure_Model!B47/Assumptions!B11</f>
+        <f>Closure_Model!B47/Exodus_Model!B8</f>
         <v/>
       </c>
     </row>
@@ -12838,11 +12838,11 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Current student population (last official SAAR end-of-year count, 2024-25)</t>
+          <t>Current student population (SAAR 2025-26 end-of-year count; the 2024-25 count of 128 anchors the capacity and cost comparisons)</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>128</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="C18" s="25" t="inlineStr">
         <is>
-          <t>Of today's 128</t>
+          <t>Of today's 115</t>
         </is>
       </c>
       <c r="D18" s="25" t="inlineStr">
@@ -14408,7 +14408,7 @@
     <row r="98">
       <c r="A98" s="21" t="inlineStr">
         <is>
-          <t>The same discipline applies to the closure direction: 128 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $847,825 to minus $11,030 with a weighted median of minus $428,627, and not the school's $2.5M gross cost.</t>
+          <t>The same discipline applies to the closure direction: 115 arriving students trigger the same class caps at the receiving schools, adding sections in several grades, which is exactly why the closure's net effect runs minus $847,825 to minus $11,030 with a weighted median of minus $428,627, and not the school's $2.5M gross cost.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Closure calculator and two-roads card open at the weighted median
The default is now the grid cell AT the weighted median ($80,279
captured, no fixed positions cut, three teachers, 154 leavers with zero
add-ons, $20,000 busing = -$427,087, the 50th percentile by
construction): the calculator opens at the middle result of all 972,
and the Shrink-to-Fit card reads -$427,087, the weighted median. The
savings-granted case (-$308,207, 82nd percentile) stays one slider-move
away as the labeled steelman, still contrasted with the superintendent's
retention stance. Grid script asserts the median cell and both ranks;
workbook Defaults B34/F34 re-pointed; report history amended; suites
re-pinned (default tax 2.6 cents, markers 50/50). Full stack green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VXyFw6349rmGg28d5ZFWpv
</commit_message>
<xml_diff>
--- a/NMES_Financial_Model.xlsx
+++ b/NMES_Financial_Model.xlsx
@@ -11190,12 +11190,12 @@
         </is>
       </c>
       <c r="B34" s="19">
-        <f>B17+C17+Closure_Model!C40+3*54479.4-63000-136*(Assumptions!B6+500-Assumptions!B62)</f>
+        <f>Closure_Model!C39+3*54479.4-Closure_Model!B42-Closure_Model!D43*(Assumptions!B6+Closure_Model!B44-Assumptions!B62)</f>
         <v/>
       </c>
       <c r="F34" s="21" t="inlineStr">
         <is>
-          <t>$127,039 kept, plus half the fixed overhead positions ($107,052, Closure_Model C40) and three teachers at $54,479.40, minus $63,000 of busing, minus the statistical median of 136 missing students at $5,126 less the $400 supplies credit: the published -$308,207, the 82nd percentile of the 972-scenario grid; the weighted median is a $427,087 loss (Closure_Model row 50)</t>
+          <t>The site calculator opens at the grid's weighted median cell: $80,279 captured (Closure_Model C39), no fixed positions cut, three teachers at $54,479.40, minus $20,000 of busing, minus the band's high 154 leavers at zero add-ons less the $400 supplies credit: the published -$427,087, the 50th percentile by construction (Closure_Model row 50). The savings-granted steelman (building sold, half the fixed positions, three teachers, median leavers) prices -$308,207 at the 82nd percentile and is one slider-move away</t>
         </is>
       </c>
     </row>
@@ -12666,7 +12666,7 @@
     <row r="50">
       <c r="A50" s="21" t="inlineStr">
         <is>
-          <t>Distribution of all 972 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, busing and missing-students levers take three values each, teachers four (0/1/2/3): 3^5 x 4 = 972. Each missing student is priced at the enacted FY2027 SEEK base of $4,626 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending; the missing-students lever prices the statistical band's quartiles (117/136/154), with the signed-survey floor of 74 (the 70 signed children spread over their twelve class cohorts, 5.83 per class, carried 12.62 effective years) kept as hard evidence below every priced leg. v5.0 lever weights: triangular 1-2-1 on every three-leg lever, uniform on teachers. Weighted median -$427,087 (the median scenario LOSES money); middle half -$518,405 to -$338,727; EVERY weighted scenario is negative, the best case still loses $9,860; range -$846,285 to -$9,860 (unweighted median -$425,053). One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
+          <t>Distribution of all 972 combinations enumerated by build/closure_grid.py: capture, fixed-position, add-ons, busing and missing-students levers take three values each, teachers four (0/1/2/3): 3^5 x 4 = 972. Each missing student is priced at the enacted FY2027 SEEK base of $4,626 plus the add-ons lever, minus the $400 of supplies that stop being spent (Assumptions row 62, the same figure the growth model charges each recruit); teacher savings appear ONLY on the teachers-cut lever, so staffing is never counted twice. The busing high leg is capped at half its bottom-up maximum ($95,000); a property-value lever priced in an interim draft is removed while the PVA records request is pending; the missing-students lever prices the statistical band's quartiles (117/136/154), with the signed-survey floor of 74 (the 70 signed children spread over their twelve class cohorts, 5.83 per class, carried 12.62 effective years) kept as hard evidence below every priced leg. v5.0 lever weights: triangular 1-2-1 on every three-leg lever, uniform on teachers. Weighted median -$427,087 (the median scenario LOSES money); middle half -$518,405 to -$338,727; EVERY weighted scenario is negative, the best case still loses $9,860; range -$846,285 to -$9,860 (unweighted median -$425,053). The site calculator opens at the cell AT the weighted median ($80,279 + 3 teachers - $20,000 busing - 154 x $4,226 = -$427,087, the 50th percentile); the savings-granted steelman (-$308,207, 82nd percentile) is retained beside it. One-time transition costs $100K-$300K in year one are additional. The v4.5 grid (5,832 scenarios, weighted median -$20,007, 55 percent negative) and the v3.9 grid (2,916, median +$21,571) are retained in the version history.</t>
         </is>
       </c>
     </row>

</xml_diff>